<commit_message>
Tiếp tục hoàn thiện giao diện ISO
</commit_message>
<xml_diff>
--- a/04-Bieu-Mau/04-FRM-400/FRM-401_Purchase_Order_Tracking_Log.xlsx
+++ b/04-Bieu-Mau/04-FRM-400/FRM-401_Purchase_Order_Tracking_Log.xlsx
@@ -778,7 +778,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="318">
+  <borders count="348">
     <border>
       <left/>
       <right/>
@@ -4175,12 +4175,367 @@
       <bottom style="medium">
         <color rgb="002C9CD7"/>
       </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="002C9CD7"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="002C9CD7"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00C5D9E8"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="002C9CD7"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="002C9CD7"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="002C9CD7"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00C5D9E8"/>
+      </left>
+      <right style="medium">
+        <color rgb="002C9CD7"/>
+      </right>
+      <top style="thin">
+        <color rgb="00C5D9E8"/>
+      </top>
+      <bottom/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="002C9CD7"/>
+      </right>
+      <top style="thin">
+        <color rgb="00C5D9E8"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00C5D9E8"/>
+      </left>
+      <right style="medium">
+        <color rgb="002C9CD7"/>
+      </right>
+      <top style="medium">
+        <color rgb="002C9CD7"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00C5D9E8"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="002C9CD7"/>
+      </right>
+      <top style="medium">
+        <color rgb="002C9CD7"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="002C9CD7"/>
+      </right>
+      <top style="medium">
+        <color rgb="002C9CD7"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00C5D9E8"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00C5D9E8"/>
+      </left>
+      <right style="medium">
+        <color rgb="002C9CD7"/>
+      </right>
+      <top style="thin">
+        <color rgb="00C5D9E8"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00C5D9E8"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="002C9CD7"/>
+      </right>
+      <top style="thin">
+        <color rgb="00C5D9E8"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00C5D9E8"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="002C9CD7"/>
+      </left>
+      <right style="thin">
+        <color rgb="00C5D9E8"/>
+      </right>
+      <top style="thin">
+        <color rgb="00C5D9E8"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="002C9CD7"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00C5D9E8"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="002C9CD7"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00C5D9E8"/>
+      </right>
+      <top style="thin">
+        <color rgb="00C5D9E8"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="002C9CD7"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="002C9CD7"/>
+      </left>
+      <right style="thin">
+        <color rgb="00C5D9E8"/>
+      </right>
+      <top style="thin">
+        <color rgb="00C5D9E8"/>
+      </top>
+      <bottom/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00C5D9E8"/>
+      </left>
+      <right style="medium">
+        <color rgb="002C9CD7"/>
+      </right>
+      <top style="thin">
+        <color rgb="00C5D9E8"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="002C9CD7"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="002C9CD7"/>
+      </right>
+      <top style="thin">
+        <color rgb="00C5D9E8"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="002C9CD7"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00C5D9E8"/>
+      </left>
+      <right style="medium">
+        <color rgb="002C9CD7"/>
+      </right>
+      <top style="medium">
+        <color rgb="002C9CD7"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="002C9CD7"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="002C9CD7"/>
+      </right>
+      <top style="medium">
+        <color rgb="002C9CD7"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="002C9CD7"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="002C9CD7"/>
+      </left>
+      <right style="medium">
+        <color rgb="002C9CD7"/>
+      </right>
+      <top/>
+      <bottom/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="002C9CD7"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="002C9CD7"/>
+      </left>
+      <right style="medium">
+        <color rgb="002C9CD7"/>
+      </right>
+      <top style="medium">
+        <color rgb="002C9CD7"/>
+      </top>
+      <bottom/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="002C9CD7"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="002C9CD7"/>
+      </left>
+      <right style="medium">
+        <color rgb="002C9CD7"/>
+      </right>
+      <top style="medium">
+        <color rgb="002C9CD7"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="002C9CD7"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="002C9CD7"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="002C9CD7"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="002C9CD7"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="002C9CD7"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="002C9CD7"/>
+      </left>
+      <right style="medium">
+        <color rgb="002C9CD7"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="002C9CD7"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="002C9CD7"/>
+      </left>
+      <right style="thin">
+        <color rgb="00C5D9E8"/>
+      </right>
+      <top style="medium">
+        <color rgb="002C9CD7"/>
+      </top>
+      <bottom/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00C5D9E8"/>
+      </right>
+      <top style="medium">
+        <color rgb="002C9CD7"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00C5D9E8"/>
+      </left>
+      <right style="medium">
+        <color rgb="002C9CD7"/>
+      </right>
+      <top style="medium">
+        <color rgb="002C9CD7"/>
+      </top>
+      <bottom/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="79" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="533">
+  <cellXfs count="574">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -5452,6 +5807,101 @@
     <xf numFmtId="0" fontId="79" fillId="0" borderId="315" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="80" fillId="0" borderId="315" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="318" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="320" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="321" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="319" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="79" fillId="4" borderId="341" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="325" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="81" fillId="4" borderId="339" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="82" fillId="47" borderId="345" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="346" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="51" fillId="4" borderId="347" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="340" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="338" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="82" fillId="47" borderId="332" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="283" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="51" fillId="4" borderId="322" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="323" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="83" fillId="4" borderId="337" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="342" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="343" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="84" fillId="4" borderId="344" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="82" fillId="47" borderId="329" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="330" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="331" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="51" fillId="4" borderId="333" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="334" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="50" borderId="341" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="336" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="319" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="324" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="326" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="284" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="327" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="328" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="330" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="333" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="334" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="48" borderId="335" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="324" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="327" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="333" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="85" fillId="4" borderId="341" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -5552,6 +6002,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -5582,6 +6035,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -5612,6 +6068,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -5642,6 +6101,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -5957,7 +6419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AN42"/>
+  <dimension ref="A1:CU42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.33" customWidth="1" min="1" max="1"/>
@@ -6008,15 +6470,15 @@
           <t>Purchase Order Tracking Log</t>
         </is>
       </c>
-      <c r="B1" s="415" t="n"/>
-      <c r="C1" s="415" t="n"/>
-      <c r="D1" s="415" t="n"/>
-      <c r="E1" s="415" t="n"/>
-      <c r="F1" s="415" t="n"/>
-      <c r="G1" s="415" t="n"/>
-      <c r="H1" s="416" t="n"/>
-      <c r="I1" s="417" t="n"/>
-      <c r="J1" s="418" t="n"/>
+      <c r="B1" s="533" t="n"/>
+      <c r="C1" s="533" t="n"/>
+      <c r="D1" s="533" t="n"/>
+      <c r="E1" s="533" t="n"/>
+      <c r="F1" s="533" t="n"/>
+      <c r="G1" s="533" t="n"/>
+      <c r="H1" s="533" t="n"/>
+      <c r="I1" s="533" t="n"/>
+      <c r="J1" s="533" t="n"/>
       <c r="K1" s="418" t="n"/>
       <c r="L1" s="418" t="n"/>
       <c r="M1" s="418" t="n"/>
@@ -6054,15 +6516,6 @@
           <t>Operational Data Sheet · FRM-401 · Owner: Controlled Owner</t>
         </is>
       </c>
-      <c r="B2" s="25" t="n"/>
-      <c r="C2" s="25" t="n"/>
-      <c r="D2" s="25" t="n"/>
-      <c r="E2" s="25" t="n"/>
-      <c r="F2" s="25" t="n"/>
-      <c r="G2" s="25" t="n"/>
-      <c r="H2" s="427" t="n"/>
-      <c r="I2" s="428" t="n"/>
-      <c r="J2" s="429" t="n"/>
       <c r="K2" s="429" t="n"/>
       <c r="L2" s="429" t="n"/>
       <c r="M2" s="429" t="n"/>
@@ -6100,15 +6553,6 @@
           <t>Controlled row-level entry. Use approved dropdowns only. Do not delete history. Refer to the FACE sheet for review context and sign-off.</t>
         </is>
       </c>
-      <c r="B3" s="25" t="n"/>
-      <c r="C3" s="25" t="n"/>
-      <c r="D3" s="25" t="n"/>
-      <c r="E3" s="25" t="n"/>
-      <c r="F3" s="25" t="n"/>
-      <c r="G3" s="25" t="n"/>
-      <c r="H3" s="427" t="n"/>
-      <c r="I3" s="428" t="n"/>
-      <c r="J3" s="429" t="n"/>
       <c r="K3" s="429" t="n"/>
       <c r="L3" s="429" t="n"/>
       <c r="M3" s="429" t="n"/>
@@ -6188,15 +6632,15 @@
           <t xml:space="preserve">  1. ACTIVE LOG TABLE</t>
         </is>
       </c>
-      <c r="B5" s="445" t="n"/>
-      <c r="C5" s="445" t="n"/>
-      <c r="D5" s="445" t="n"/>
-      <c r="E5" s="445" t="n"/>
-      <c r="F5" s="445" t="n"/>
-      <c r="G5" s="445" t="n"/>
-      <c r="H5" s="446" t="n"/>
-      <c r="I5" s="447" t="n"/>
-      <c r="J5" s="448" t="n"/>
+      <c r="B5" s="534" t="n"/>
+      <c r="C5" s="534" t="n"/>
+      <c r="D5" s="534" t="n"/>
+      <c r="E5" s="534" t="n"/>
+      <c r="F5" s="534" t="n"/>
+      <c r="G5" s="534" t="n"/>
+      <c r="H5" s="534" t="n"/>
+      <c r="I5" s="534" t="n"/>
+      <c r="J5" s="534" t="n"/>
       <c r="K5" s="448" t="n"/>
       <c r="L5" s="448" t="n"/>
       <c r="M5" s="448" t="n"/>
@@ -7708,15 +8152,15 @@
           <t xml:space="preserve">  2. PERIODIC REVIEW / CLOSEOUT</t>
         </is>
       </c>
-      <c r="B38" s="473" t="n"/>
-      <c r="C38" s="473" t="n"/>
-      <c r="D38" s="473" t="n"/>
-      <c r="E38" s="473" t="n"/>
-      <c r="F38" s="473" t="n"/>
-      <c r="G38" s="473" t="n"/>
-      <c r="H38" s="473" t="n"/>
-      <c r="I38" s="473" t="n"/>
-      <c r="J38" s="473" t="n"/>
+      <c r="B38" s="535" t="n"/>
+      <c r="C38" s="535" t="n"/>
+      <c r="D38" s="535" t="n"/>
+      <c r="E38" s="535" t="n"/>
+      <c r="F38" s="535" t="n"/>
+      <c r="G38" s="535" t="n"/>
+      <c r="H38" s="535" t="n"/>
+      <c r="I38" s="535" t="n"/>
+      <c r="J38" s="535" t="n"/>
       <c r="K38" s="473" t="n"/>
       <c r="L38" s="473" t="n"/>
       <c r="M38" s="473" t="n"/>
@@ -7754,19 +8198,19 @@
           <t>Review Date</t>
         </is>
       </c>
-      <c r="B39" s="462" t="n"/>
+      <c r="B39" s="536" t="n"/>
       <c r="C39" s="476" t="inlineStr"/>
-      <c r="D39" s="462" t="n"/>
-      <c r="E39" s="462" t="n"/>
+      <c r="D39" s="536" t="n"/>
+      <c r="E39" s="536" t="n"/>
       <c r="F39" s="477" t="inlineStr">
         <is>
           <t>Reviewer</t>
         </is>
       </c>
-      <c r="G39" s="462" t="n"/>
+      <c r="G39" s="536" t="n"/>
       <c r="H39" s="476" t="inlineStr"/>
-      <c r="I39" s="462" t="n"/>
-      <c r="J39" s="462" t="n"/>
+      <c r="I39" s="536" t="n"/>
+      <c r="J39" s="536" t="n"/>
       <c r="K39" s="478" t="n"/>
       <c r="L39" s="462" t="n"/>
       <c r="M39" s="462" t="n"/>
@@ -7804,19 +8248,19 @@
           <t>Open Items / Exceptions</t>
         </is>
       </c>
-      <c r="B40" s="349" t="n"/>
+      <c r="B40" s="408" t="n"/>
       <c r="C40" s="480" t="inlineStr"/>
-      <c r="D40" s="349" t="n"/>
-      <c r="E40" s="349" t="n"/>
+      <c r="D40" s="408" t="n"/>
+      <c r="E40" s="408" t="n"/>
       <c r="F40" s="481" t="inlineStr">
         <is>
           <t>Final Status</t>
         </is>
       </c>
-      <c r="G40" s="349" t="n"/>
+      <c r="G40" s="408" t="n"/>
       <c r="H40" s="480" t="inlineStr"/>
-      <c r="I40" s="349" t="n"/>
-      <c r="J40" s="349" t="n"/>
+      <c r="I40" s="408" t="n"/>
+      <c r="J40" s="408" t="n"/>
       <c r="K40" s="482" t="n"/>
       <c r="L40" s="360" t="n"/>
       <c r="M40" s="360" t="n"/>
@@ -7896,15 +8340,15 @@
           <t>NOTICE: Complete in English. Do not back-date, delete history, or overwrite a closed row without a controlled supplemental entry. Review / sign-off context remains on sheet PO_EXCEPTION_LOG. Exception-log only. Do not use this workbook as an Epicor replacement PO tracker.</t>
         </is>
       </c>
-      <c r="B42" s="473" t="n"/>
-      <c r="C42" s="473" t="n"/>
-      <c r="D42" s="473" t="n"/>
-      <c r="E42" s="473" t="n"/>
-      <c r="F42" s="473" t="n"/>
-      <c r="G42" s="473" t="n"/>
-      <c r="H42" s="473" t="n"/>
-      <c r="I42" s="473" t="n"/>
-      <c r="J42" s="473" t="n"/>
+      <c r="B42" s="535" t="n"/>
+      <c r="C42" s="535" t="n"/>
+      <c r="D42" s="535" t="n"/>
+      <c r="E42" s="535" t="n"/>
+      <c r="F42" s="535" t="n"/>
+      <c r="G42" s="535" t="n"/>
+      <c r="H42" s="535" t="n"/>
+      <c r="I42" s="535" t="n"/>
+      <c r="J42" s="535" t="n"/>
       <c r="K42" s="473" t="n"/>
       <c r="L42" s="473" t="n"/>
       <c r="M42" s="473" t="n"/>
@@ -7983,7 +8427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BD32"/>
+  <dimension ref="A1:CU32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.33" customWidth="1" min="1" max="1"/>
@@ -8045,326 +8489,212 @@
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
-      <c r="A1" s="483" t="n"/>
-      <c r="B1" s="415" t="n"/>
-      <c r="C1" s="415" t="n"/>
-      <c r="D1" s="415" t="n"/>
-      <c r="E1" s="415" t="n"/>
-      <c r="F1" s="415" t="n"/>
-      <c r="G1" s="415" t="n"/>
-      <c r="H1" s="415" t="n"/>
-      <c r="I1" s="415" t="n"/>
-      <c r="J1" s="415" t="n"/>
-      <c r="K1" s="416" t="n"/>
-      <c r="L1" s="417" t="inlineStr">
+      <c r="A1" s="537" t="n"/>
+      <c r="B1" s="533" t="n"/>
+      <c r="C1" s="533" t="n"/>
+      <c r="D1" s="533" t="n"/>
+      <c r="E1" s="533" t="n"/>
+      <c r="F1" s="533" t="n"/>
+      <c r="G1" s="533" t="n"/>
+      <c r="H1" s="533" t="n"/>
+      <c r="I1" s="533" t="n"/>
+      <c r="J1" s="533" t="n"/>
+      <c r="K1" s="538" t="n"/>
+      <c r="L1" s="539" t="inlineStr">
         <is>
           <t>Purchase Order Tracking Log</t>
         </is>
       </c>
-      <c r="M1" s="418" t="n"/>
-      <c r="N1" s="418" t="n"/>
-      <c r="O1" s="418" t="n"/>
-      <c r="P1" s="418" t="n"/>
-      <c r="Q1" s="418" t="n"/>
-      <c r="R1" s="418" t="n"/>
-      <c r="S1" s="418" t="n"/>
-      <c r="T1" s="418" t="n"/>
-      <c r="U1" s="418" t="n"/>
-      <c r="V1" s="418" t="n"/>
-      <c r="W1" s="418" t="n"/>
-      <c r="X1" s="418" t="n"/>
-      <c r="Y1" s="418" t="n"/>
-      <c r="Z1" s="418" t="n"/>
-      <c r="AA1" s="418" t="n"/>
-      <c r="AB1" s="418" t="n"/>
-      <c r="AC1" s="418" t="n"/>
-      <c r="AD1" s="418" t="n"/>
-      <c r="AE1" s="418" t="n"/>
-      <c r="AF1" s="418" t="n"/>
-      <c r="AG1" s="418" t="n"/>
-      <c r="AH1" s="418" t="n"/>
-      <c r="AI1" s="418" t="n"/>
-      <c r="AJ1" s="418" t="n"/>
-      <c r="AK1" s="418" t="n"/>
-      <c r="AL1" s="418" t="n"/>
-      <c r="AM1" s="418" t="n"/>
-      <c r="AN1" s="418" t="n"/>
-      <c r="AO1" s="418" t="n"/>
-      <c r="AP1" s="419" t="n"/>
-      <c r="AQ1" s="420" t="n"/>
-      <c r="AR1" s="421" t="n"/>
-      <c r="AS1" s="421" t="n"/>
-      <c r="AT1" s="421" t="n"/>
-      <c r="AU1" s="421" t="n"/>
-      <c r="AV1" s="422" t="n"/>
-      <c r="AW1" s="423" t="inlineStr">
+      <c r="M1" s="533" t="n"/>
+      <c r="N1" s="533" t="n"/>
+      <c r="O1" s="533" t="n"/>
+      <c r="P1" s="533" t="n"/>
+      <c r="Q1" s="533" t="n"/>
+      <c r="R1" s="533" t="n"/>
+      <c r="S1" s="533" t="n"/>
+      <c r="T1" s="533" t="n"/>
+      <c r="U1" s="533" t="n"/>
+      <c r="V1" s="533" t="n"/>
+      <c r="W1" s="533" t="n"/>
+      <c r="X1" s="533" t="n"/>
+      <c r="Y1" s="533" t="n"/>
+      <c r="Z1" s="533" t="n"/>
+      <c r="AA1" s="533" t="n"/>
+      <c r="AB1" s="533" t="n"/>
+      <c r="AC1" s="533" t="n"/>
+      <c r="AD1" s="533" t="n"/>
+      <c r="AE1" s="533" t="n"/>
+      <c r="AF1" s="533" t="n"/>
+      <c r="AG1" s="533" t="n"/>
+      <c r="AH1" s="533" t="n"/>
+      <c r="AI1" s="533" t="n"/>
+      <c r="AJ1" s="533" t="n"/>
+      <c r="AK1" s="533" t="n"/>
+      <c r="AL1" s="533" t="n"/>
+      <c r="AM1" s="533" t="n"/>
+      <c r="AN1" s="533" t="n"/>
+      <c r="AO1" s="533" t="n"/>
+      <c r="AP1" s="538" t="n"/>
+      <c r="AQ1" s="540" t="n"/>
+      <c r="AR1" s="533" t="n"/>
+      <c r="AS1" s="533" t="n"/>
+      <c r="AT1" s="533" t="n"/>
+      <c r="AU1" s="533" t="n"/>
+      <c r="AV1" s="541" t="n"/>
+      <c r="AW1" s="542" t="inlineStr">
         <is>
           <t>FRM-401</t>
         </is>
       </c>
-      <c r="AX1" s="424" t="n"/>
-      <c r="AY1" s="424" t="n"/>
-      <c r="AZ1" s="424" t="n"/>
-      <c r="BA1" s="424" t="n"/>
-      <c r="BB1" s="424" t="n"/>
-      <c r="BC1" s="424" t="n"/>
-      <c r="BD1" s="425" t="n"/>
+      <c r="AX1" s="533" t="n"/>
+      <c r="AY1" s="533" t="n"/>
+      <c r="AZ1" s="533" t="n"/>
+      <c r="BA1" s="533" t="n"/>
+      <c r="BB1" s="533" t="n"/>
+      <c r="BC1" s="533" t="n"/>
+      <c r="BD1" s="538" t="n"/>
     </row>
     <row r="2" ht="15" customHeight="1">
-      <c r="A2" s="484" t="n"/>
-      <c r="B2" s="25" t="n"/>
-      <c r="C2" s="25" t="n"/>
-      <c r="D2" s="25" t="n"/>
-      <c r="E2" s="25" t="n"/>
-      <c r="F2" s="25" t="n"/>
-      <c r="G2" s="25" t="n"/>
-      <c r="H2" s="25" t="n"/>
-      <c r="I2" s="25" t="n"/>
-      <c r="J2" s="25" t="n"/>
-      <c r="K2" s="427" t="n"/>
-      <c r="L2" s="428" t="n"/>
-      <c r="M2" s="429" t="n"/>
-      <c r="N2" s="429" t="n"/>
-      <c r="O2" s="429" t="n"/>
-      <c r="P2" s="429" t="n"/>
-      <c r="Q2" s="429" t="n"/>
-      <c r="R2" s="429" t="n"/>
-      <c r="S2" s="429" t="n"/>
-      <c r="T2" s="429" t="n"/>
-      <c r="U2" s="429" t="n"/>
-      <c r="V2" s="429" t="n"/>
-      <c r="W2" s="429" t="n"/>
-      <c r="X2" s="429" t="n"/>
-      <c r="Y2" s="429" t="n"/>
-      <c r="Z2" s="429" t="n"/>
-      <c r="AA2" s="429" t="n"/>
-      <c r="AB2" s="429" t="n"/>
-      <c r="AC2" s="429" t="n"/>
-      <c r="AD2" s="429" t="n"/>
-      <c r="AE2" s="429" t="n"/>
-      <c r="AF2" s="429" t="n"/>
-      <c r="AG2" s="429" t="n"/>
-      <c r="AH2" s="429" t="n"/>
-      <c r="AI2" s="429" t="n"/>
-      <c r="AJ2" s="429" t="n"/>
-      <c r="AK2" s="429" t="n"/>
-      <c r="AL2" s="429" t="n"/>
-      <c r="AM2" s="429" t="n"/>
-      <c r="AN2" s="429" t="n"/>
-      <c r="AO2" s="429" t="n"/>
-      <c r="AP2" s="430" t="n"/>
-      <c r="AQ2" s="431" t="n"/>
-      <c r="AR2" s="432" t="n"/>
-      <c r="AS2" s="432" t="n"/>
-      <c r="AT2" s="432" t="n"/>
-      <c r="AU2" s="432" t="n"/>
-      <c r="AV2" s="433" t="n"/>
-      <c r="AW2" s="434" t="inlineStr">
+      <c r="A2" s="543" t="n"/>
+      <c r="K2" s="544" t="n"/>
+      <c r="L2" s="543" t="n"/>
+      <c r="AP2" s="544" t="n"/>
+      <c r="AQ2" s="545" t="n"/>
+      <c r="AR2" s="410" t="n"/>
+      <c r="AS2" s="410" t="n"/>
+      <c r="AT2" s="410" t="n"/>
+      <c r="AU2" s="410" t="n"/>
+      <c r="AV2" s="546" t="n"/>
+      <c r="AW2" s="547" t="inlineStr">
         <is>
           <t>V0</t>
         </is>
       </c>
-      <c r="AX2" s="435" t="n"/>
-      <c r="AY2" s="435" t="n"/>
-      <c r="AZ2" s="435" t="n"/>
-      <c r="BA2" s="435" t="n"/>
-      <c r="BB2" s="435" t="n"/>
-      <c r="BC2" s="435" t="n"/>
-      <c r="BD2" s="436" t="n"/>
+      <c r="AX2" s="410" t="n"/>
+      <c r="AY2" s="410" t="n"/>
+      <c r="AZ2" s="410" t="n"/>
+      <c r="BA2" s="410" t="n"/>
+      <c r="BB2" s="410" t="n"/>
+      <c r="BC2" s="410" t="n"/>
+      <c r="BD2" s="548" t="n"/>
     </row>
     <row r="3" ht="15" customHeight="1">
-      <c r="A3" s="484" t="n"/>
-      <c r="B3" s="25" t="n"/>
-      <c r="C3" s="25" t="n"/>
-      <c r="D3" s="25" t="n"/>
-      <c r="E3" s="25" t="n"/>
-      <c r="F3" s="25" t="n"/>
-      <c r="G3" s="25" t="n"/>
-      <c r="H3" s="25" t="n"/>
-      <c r="I3" s="25" t="n"/>
-      <c r="J3" s="25" t="n"/>
-      <c r="K3" s="427" t="n"/>
-      <c r="L3" s="428" t="n"/>
-      <c r="M3" s="429" t="n"/>
-      <c r="N3" s="429" t="n"/>
-      <c r="O3" s="429" t="n"/>
-      <c r="P3" s="429" t="n"/>
-      <c r="Q3" s="429" t="n"/>
-      <c r="R3" s="429" t="n"/>
-      <c r="S3" s="429" t="n"/>
-      <c r="T3" s="429" t="n"/>
-      <c r="U3" s="429" t="n"/>
-      <c r="V3" s="429" t="n"/>
-      <c r="W3" s="429" t="n"/>
-      <c r="X3" s="429" t="n"/>
-      <c r="Y3" s="429" t="n"/>
-      <c r="Z3" s="429" t="n"/>
-      <c r="AA3" s="429" t="n"/>
-      <c r="AB3" s="429" t="n"/>
-      <c r="AC3" s="429" t="n"/>
-      <c r="AD3" s="429" t="n"/>
-      <c r="AE3" s="429" t="n"/>
-      <c r="AF3" s="429" t="n"/>
-      <c r="AG3" s="429" t="n"/>
-      <c r="AH3" s="429" t="n"/>
-      <c r="AI3" s="429" t="n"/>
-      <c r="AJ3" s="429" t="n"/>
-      <c r="AK3" s="429" t="n"/>
-      <c r="AL3" s="429" t="n"/>
-      <c r="AM3" s="429" t="n"/>
-      <c r="AN3" s="429" t="n"/>
-      <c r="AO3" s="429" t="n"/>
-      <c r="AP3" s="430" t="n"/>
-      <c r="AQ3" s="431" t="n"/>
-      <c r="AR3" s="432" t="n"/>
-      <c r="AS3" s="432" t="n"/>
-      <c r="AT3" s="432" t="n"/>
-      <c r="AU3" s="432" t="n"/>
-      <c r="AV3" s="433" t="n"/>
-      <c r="AW3" s="434" t="inlineStr">
+      <c r="A3" s="543" t="n"/>
+      <c r="K3" s="544" t="n"/>
+      <c r="L3" s="543" t="n"/>
+      <c r="AP3" s="544" t="n"/>
+      <c r="AQ3" s="545" t="n"/>
+      <c r="AR3" s="410" t="n"/>
+      <c r="AS3" s="410" t="n"/>
+      <c r="AT3" s="410" t="n"/>
+      <c r="AU3" s="410" t="n"/>
+      <c r="AV3" s="546" t="n"/>
+      <c r="AW3" s="547" t="inlineStr">
         <is>
           <t>YYYY-MM-DD</t>
         </is>
       </c>
-      <c r="AX3" s="435" t="n"/>
-      <c r="AY3" s="435" t="n"/>
-      <c r="AZ3" s="435" t="n"/>
-      <c r="BA3" s="435" t="n"/>
-      <c r="BB3" s="435" t="n"/>
-      <c r="BC3" s="435" t="n"/>
-      <c r="BD3" s="436" t="n"/>
+      <c r="AX3" s="410" t="n"/>
+      <c r="AY3" s="410" t="n"/>
+      <c r="AZ3" s="410" t="n"/>
+      <c r="BA3" s="410" t="n"/>
+      <c r="BB3" s="410" t="n"/>
+      <c r="BC3" s="410" t="n"/>
+      <c r="BD3" s="548" t="n"/>
     </row>
     <row r="4" ht="15" customHeight="1">
-      <c r="A4" s="484" t="n"/>
-      <c r="B4" s="25" t="n"/>
-      <c r="C4" s="25" t="n"/>
-      <c r="D4" s="25" t="n"/>
-      <c r="E4" s="25" t="n"/>
-      <c r="F4" s="25" t="n"/>
-      <c r="G4" s="25" t="n"/>
-      <c r="H4" s="25" t="n"/>
-      <c r="I4" s="25" t="n"/>
-      <c r="J4" s="25" t="n"/>
-      <c r="K4" s="427" t="n"/>
-      <c r="L4" s="441" t="inlineStr">
+      <c r="A4" s="543" t="n"/>
+      <c r="K4" s="544" t="n"/>
+      <c r="L4" s="549" t="inlineStr">
         <is>
           <t>Quality Management System · Controlled Document</t>
         </is>
       </c>
-      <c r="M4" s="442" t="n"/>
-      <c r="N4" s="442" t="n"/>
-      <c r="O4" s="442" t="n"/>
-      <c r="P4" s="442" t="n"/>
-      <c r="Q4" s="442" t="n"/>
-      <c r="R4" s="442" t="n"/>
-      <c r="S4" s="442" t="n"/>
-      <c r="T4" s="442" t="n"/>
-      <c r="U4" s="442" t="n"/>
-      <c r="V4" s="442" t="n"/>
-      <c r="W4" s="442" t="n"/>
-      <c r="X4" s="442" t="n"/>
-      <c r="Y4" s="442" t="n"/>
-      <c r="Z4" s="442" t="n"/>
-      <c r="AA4" s="442" t="n"/>
-      <c r="AB4" s="442" t="n"/>
-      <c r="AC4" s="442" t="n"/>
-      <c r="AD4" s="442" t="n"/>
-      <c r="AE4" s="442" t="n"/>
-      <c r="AF4" s="442" t="n"/>
-      <c r="AG4" s="442" t="n"/>
-      <c r="AH4" s="442" t="n"/>
-      <c r="AI4" s="442" t="n"/>
-      <c r="AJ4" s="442" t="n"/>
-      <c r="AK4" s="442" t="n"/>
-      <c r="AL4" s="442" t="n"/>
-      <c r="AM4" s="442" t="n"/>
-      <c r="AN4" s="442" t="n"/>
-      <c r="AO4" s="442" t="n"/>
-      <c r="AP4" s="443" t="n"/>
-      <c r="AQ4" s="431" t="n"/>
-      <c r="AR4" s="432" t="n"/>
-      <c r="AS4" s="432" t="n"/>
-      <c r="AT4" s="432" t="n"/>
-      <c r="AU4" s="432" t="n"/>
-      <c r="AV4" s="433" t="n"/>
-      <c r="AW4" s="434" t="inlineStr">
+      <c r="AP4" s="544" t="n"/>
+      <c r="AQ4" s="545" t="n"/>
+      <c r="AR4" s="410" t="n"/>
+      <c r="AS4" s="410" t="n"/>
+      <c r="AT4" s="410" t="n"/>
+      <c r="AU4" s="410" t="n"/>
+      <c r="AV4" s="546" t="n"/>
+      <c r="AW4" s="547" t="inlineStr">
         <is>
           <t>Purchasing + QA</t>
         </is>
       </c>
-      <c r="AX4" s="435" t="n"/>
-      <c r="AY4" s="435" t="n"/>
-      <c r="AZ4" s="435" t="n"/>
-      <c r="BA4" s="435" t="n"/>
-      <c r="BB4" s="435" t="n"/>
-      <c r="BC4" s="435" t="n"/>
-      <c r="BD4" s="436" t="n"/>
+      <c r="AX4" s="410" t="n"/>
+      <c r="AY4" s="410" t="n"/>
+      <c r="AZ4" s="410" t="n"/>
+      <c r="BA4" s="410" t="n"/>
+      <c r="BB4" s="410" t="n"/>
+      <c r="BC4" s="410" t="n"/>
+      <c r="BD4" s="548" t="n"/>
     </row>
     <row r="5" ht="15" customHeight="1">
-      <c r="A5" s="485" t="n"/>
-      <c r="B5" s="445" t="n"/>
-      <c r="C5" s="445" t="n"/>
-      <c r="D5" s="445" t="n"/>
-      <c r="E5" s="445" t="n"/>
-      <c r="F5" s="445" t="n"/>
-      <c r="G5" s="445" t="n"/>
-      <c r="H5" s="445" t="n"/>
-      <c r="I5" s="445" t="n"/>
-      <c r="J5" s="445" t="n"/>
-      <c r="K5" s="446" t="n"/>
-      <c r="L5" s="447" t="inlineStr">
+      <c r="A5" s="550" t="n"/>
+      <c r="B5" s="534" t="n"/>
+      <c r="C5" s="534" t="n"/>
+      <c r="D5" s="534" t="n"/>
+      <c r="E5" s="534" t="n"/>
+      <c r="F5" s="534" t="n"/>
+      <c r="G5" s="534" t="n"/>
+      <c r="H5" s="534" t="n"/>
+      <c r="I5" s="534" t="n"/>
+      <c r="J5" s="534" t="n"/>
+      <c r="K5" s="551" t="n"/>
+      <c r="L5" s="552" t="inlineStr">
         <is>
           <t>HESEM Engineering · ISO 9001 / AS9100 · Semiconductor Equipment Parts</t>
         </is>
       </c>
-      <c r="M5" s="448" t="n"/>
-      <c r="N5" s="448" t="n"/>
-      <c r="O5" s="448" t="n"/>
-      <c r="P5" s="448" t="n"/>
-      <c r="Q5" s="448" t="n"/>
-      <c r="R5" s="448" t="n"/>
-      <c r="S5" s="448" t="n"/>
-      <c r="T5" s="448" t="n"/>
-      <c r="U5" s="448" t="n"/>
-      <c r="V5" s="448" t="n"/>
-      <c r="W5" s="448" t="n"/>
-      <c r="X5" s="448" t="n"/>
-      <c r="Y5" s="448" t="n"/>
-      <c r="Z5" s="448" t="n"/>
-      <c r="AA5" s="448" t="n"/>
-      <c r="AB5" s="448" t="n"/>
-      <c r="AC5" s="448" t="n"/>
-      <c r="AD5" s="448" t="n"/>
-      <c r="AE5" s="448" t="n"/>
-      <c r="AF5" s="448" t="n"/>
-      <c r="AG5" s="448" t="n"/>
-      <c r="AH5" s="448" t="n"/>
-      <c r="AI5" s="448" t="n"/>
-      <c r="AJ5" s="448" t="n"/>
-      <c r="AK5" s="448" t="n"/>
-      <c r="AL5" s="448" t="n"/>
-      <c r="AM5" s="448" t="n"/>
-      <c r="AN5" s="448" t="n"/>
-      <c r="AO5" s="448" t="n"/>
-      <c r="AP5" s="449" t="n"/>
-      <c r="AQ5" s="450" t="n"/>
-      <c r="AR5" s="451" t="n"/>
-      <c r="AS5" s="451" t="n"/>
-      <c r="AT5" s="451" t="n"/>
-      <c r="AU5" s="451" t="n"/>
-      <c r="AV5" s="452" t="n"/>
-      <c r="AW5" s="453" t="inlineStr">
+      <c r="M5" s="534" t="n"/>
+      <c r="N5" s="534" t="n"/>
+      <c r="O5" s="534" t="n"/>
+      <c r="P5" s="534" t="n"/>
+      <c r="Q5" s="534" t="n"/>
+      <c r="R5" s="534" t="n"/>
+      <c r="S5" s="534" t="n"/>
+      <c r="T5" s="534" t="n"/>
+      <c r="U5" s="534" t="n"/>
+      <c r="V5" s="534" t="n"/>
+      <c r="W5" s="534" t="n"/>
+      <c r="X5" s="534" t="n"/>
+      <c r="Y5" s="534" t="n"/>
+      <c r="Z5" s="534" t="n"/>
+      <c r="AA5" s="534" t="n"/>
+      <c r="AB5" s="534" t="n"/>
+      <c r="AC5" s="534" t="n"/>
+      <c r="AD5" s="534" t="n"/>
+      <c r="AE5" s="534" t="n"/>
+      <c r="AF5" s="534" t="n"/>
+      <c r="AG5" s="534" t="n"/>
+      <c r="AH5" s="534" t="n"/>
+      <c r="AI5" s="534" t="n"/>
+      <c r="AJ5" s="534" t="n"/>
+      <c r="AK5" s="534" t="n"/>
+      <c r="AL5" s="534" t="n"/>
+      <c r="AM5" s="534" t="n"/>
+      <c r="AN5" s="534" t="n"/>
+      <c r="AO5" s="534" t="n"/>
+      <c r="AP5" s="551" t="n"/>
+      <c r="AQ5" s="553" t="n"/>
+      <c r="AR5" s="554" t="n"/>
+      <c r="AS5" s="554" t="n"/>
+      <c r="AT5" s="554" t="n"/>
+      <c r="AU5" s="554" t="n"/>
+      <c r="AV5" s="555" t="n"/>
+      <c r="AW5" s="556" t="inlineStr">
         <is>
           <t>General Manager</t>
         </is>
       </c>
-      <c r="AX5" s="454" t="n"/>
-      <c r="AY5" s="454" t="n"/>
-      <c r="AZ5" s="454" t="n"/>
-      <c r="BA5" s="454" t="n"/>
-      <c r="BB5" s="454" t="n"/>
-      <c r="BC5" s="454" t="n"/>
-      <c r="BD5" s="455" t="n"/>
+      <c r="AX5" s="554" t="n"/>
+      <c r="AY5" s="554" t="n"/>
+      <c r="AZ5" s="554" t="n"/>
+      <c r="BA5" s="554" t="n"/>
+      <c r="BB5" s="554" t="n"/>
+      <c r="BC5" s="554" t="n"/>
+      <c r="BD5" s="557" t="n"/>
     </row>
     <row r="6" ht="1.5" customHeight="1">
       <c r="A6" s="486" t="n"/>
@@ -8425,66 +8755,66 @@
       <c r="BD6" s="486" t="n"/>
     </row>
     <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="472" t="inlineStr">
+      <c r="A7" s="558" t="inlineStr">
         <is>
           <t xml:space="preserve">  1. SCOPE / REVIEW CONTEXT</t>
         </is>
       </c>
-      <c r="B7" s="473" t="n"/>
-      <c r="C7" s="473" t="n"/>
-      <c r="D7" s="473" t="n"/>
-      <c r="E7" s="473" t="n"/>
-      <c r="F7" s="473" t="n"/>
-      <c r="G7" s="473" t="n"/>
-      <c r="H7" s="473" t="n"/>
-      <c r="I7" s="473" t="n"/>
-      <c r="J7" s="473" t="n"/>
-      <c r="K7" s="473" t="n"/>
-      <c r="L7" s="473" t="n"/>
-      <c r="M7" s="473" t="n"/>
-      <c r="N7" s="473" t="n"/>
-      <c r="O7" s="473" t="n"/>
-      <c r="P7" s="473" t="n"/>
-      <c r="Q7" s="473" t="n"/>
-      <c r="R7" s="473" t="n"/>
-      <c r="S7" s="473" t="n"/>
-      <c r="T7" s="473" t="n"/>
-      <c r="U7" s="473" t="n"/>
-      <c r="V7" s="473" t="n"/>
-      <c r="W7" s="473" t="n"/>
-      <c r="X7" s="473" t="n"/>
-      <c r="Y7" s="473" t="n"/>
-      <c r="Z7" s="473" t="n"/>
-      <c r="AA7" s="473" t="n"/>
-      <c r="AB7" s="473" t="n"/>
-      <c r="AC7" s="473" t="n"/>
-      <c r="AD7" s="473" t="n"/>
-      <c r="AE7" s="473" t="n"/>
-      <c r="AF7" s="473" t="n"/>
-      <c r="AG7" s="473" t="n"/>
-      <c r="AH7" s="473" t="n"/>
-      <c r="AI7" s="473" t="n"/>
-      <c r="AJ7" s="473" t="n"/>
-      <c r="AK7" s="473" t="n"/>
-      <c r="AL7" s="473" t="n"/>
-      <c r="AM7" s="473" t="n"/>
-      <c r="AN7" s="473" t="n"/>
-      <c r="AO7" s="473" t="n"/>
-      <c r="AP7" s="473" t="n"/>
-      <c r="AQ7" s="473" t="n"/>
-      <c r="AR7" s="473" t="n"/>
-      <c r="AS7" s="473" t="n"/>
-      <c r="AT7" s="473" t="n"/>
-      <c r="AU7" s="473" t="n"/>
-      <c r="AV7" s="473" t="n"/>
-      <c r="AW7" s="473" t="n"/>
-      <c r="AX7" s="473" t="n"/>
-      <c r="AY7" s="473" t="n"/>
-      <c r="AZ7" s="473" t="n"/>
-      <c r="BA7" s="473" t="n"/>
-      <c r="BB7" s="473" t="n"/>
-      <c r="BC7" s="473" t="n"/>
-      <c r="BD7" s="474" t="n"/>
+      <c r="B7" s="535" t="n"/>
+      <c r="C7" s="535" t="n"/>
+      <c r="D7" s="535" t="n"/>
+      <c r="E7" s="535" t="n"/>
+      <c r="F7" s="535" t="n"/>
+      <c r="G7" s="535" t="n"/>
+      <c r="H7" s="535" t="n"/>
+      <c r="I7" s="535" t="n"/>
+      <c r="J7" s="535" t="n"/>
+      <c r="K7" s="535" t="n"/>
+      <c r="L7" s="535" t="n"/>
+      <c r="M7" s="535" t="n"/>
+      <c r="N7" s="535" t="n"/>
+      <c r="O7" s="535" t="n"/>
+      <c r="P7" s="535" t="n"/>
+      <c r="Q7" s="535" t="n"/>
+      <c r="R7" s="535" t="n"/>
+      <c r="S7" s="535" t="n"/>
+      <c r="T7" s="535" t="n"/>
+      <c r="U7" s="535" t="n"/>
+      <c r="V7" s="535" t="n"/>
+      <c r="W7" s="535" t="n"/>
+      <c r="X7" s="535" t="n"/>
+      <c r="Y7" s="535" t="n"/>
+      <c r="Z7" s="535" t="n"/>
+      <c r="AA7" s="535" t="n"/>
+      <c r="AB7" s="535" t="n"/>
+      <c r="AC7" s="535" t="n"/>
+      <c r="AD7" s="535" t="n"/>
+      <c r="AE7" s="535" t="n"/>
+      <c r="AF7" s="535" t="n"/>
+      <c r="AG7" s="535" t="n"/>
+      <c r="AH7" s="535" t="n"/>
+      <c r="AI7" s="535" t="n"/>
+      <c r="AJ7" s="535" t="n"/>
+      <c r="AK7" s="535" t="n"/>
+      <c r="AL7" s="535" t="n"/>
+      <c r="AM7" s="535" t="n"/>
+      <c r="AN7" s="535" t="n"/>
+      <c r="AO7" s="535" t="n"/>
+      <c r="AP7" s="535" t="n"/>
+      <c r="AQ7" s="535" t="n"/>
+      <c r="AR7" s="535" t="n"/>
+      <c r="AS7" s="535" t="n"/>
+      <c r="AT7" s="535" t="n"/>
+      <c r="AU7" s="535" t="n"/>
+      <c r="AV7" s="535" t="n"/>
+      <c r="AW7" s="535" t="n"/>
+      <c r="AX7" s="535" t="n"/>
+      <c r="AY7" s="535" t="n"/>
+      <c r="AZ7" s="535" t="n"/>
+      <c r="BA7" s="535" t="n"/>
+      <c r="BB7" s="535" t="n"/>
+      <c r="BC7" s="535" t="n"/>
+      <c r="BD7" s="559" t="n"/>
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="475" t="inlineStr">
@@ -8492,65 +8822,65 @@
           <t>PO Exception Log ID</t>
         </is>
       </c>
-      <c r="B8" s="462" t="n"/>
-      <c r="C8" s="462" t="n"/>
-      <c r="D8" s="462" t="n"/>
-      <c r="E8" s="462" t="n"/>
-      <c r="F8" s="462" t="n"/>
-      <c r="G8" s="462" t="n"/>
-      <c r="H8" s="462" t="n"/>
-      <c r="I8" s="462" t="n"/>
-      <c r="J8" s="462" t="n"/>
+      <c r="B8" s="536" t="n"/>
+      <c r="C8" s="536" t="n"/>
+      <c r="D8" s="536" t="n"/>
+      <c r="E8" s="536" t="n"/>
+      <c r="F8" s="536" t="n"/>
+      <c r="G8" s="536" t="n"/>
+      <c r="H8" s="536" t="n"/>
+      <c r="I8" s="536" t="n"/>
+      <c r="J8" s="536" t="n"/>
       <c r="K8" s="487" t="n"/>
-      <c r="L8" s="488" t="n"/>
-      <c r="M8" s="488" t="n"/>
-      <c r="N8" s="488" t="n"/>
-      <c r="O8" s="488" t="n"/>
-      <c r="P8" s="488" t="n"/>
-      <c r="Q8" s="488" t="n"/>
-      <c r="R8" s="488" t="n"/>
-      <c r="S8" s="488" t="n"/>
-      <c r="T8" s="488" t="n"/>
-      <c r="U8" s="488" t="n"/>
-      <c r="V8" s="488" t="n"/>
-      <c r="W8" s="488" t="n"/>
-      <c r="X8" s="488" t="n"/>
-      <c r="Y8" s="488" t="n"/>
-      <c r="Z8" s="488" t="n"/>
-      <c r="AA8" s="488" t="n"/>
-      <c r="AB8" s="488" t="n"/>
+      <c r="L8" s="560" t="n"/>
+      <c r="M8" s="560" t="n"/>
+      <c r="N8" s="560" t="n"/>
+      <c r="O8" s="560" t="n"/>
+      <c r="P8" s="560" t="n"/>
+      <c r="Q8" s="560" t="n"/>
+      <c r="R8" s="560" t="n"/>
+      <c r="S8" s="560" t="n"/>
+      <c r="T8" s="560" t="n"/>
+      <c r="U8" s="560" t="n"/>
+      <c r="V8" s="560" t="n"/>
+      <c r="W8" s="560" t="n"/>
+      <c r="X8" s="560" t="n"/>
+      <c r="Y8" s="560" t="n"/>
+      <c r="Z8" s="560" t="n"/>
+      <c r="AA8" s="560" t="n"/>
+      <c r="AB8" s="560" t="n"/>
       <c r="AC8" s="477" t="inlineStr">
         <is>
           <t>Exception Status</t>
         </is>
       </c>
-      <c r="AD8" s="462" t="n"/>
-      <c r="AE8" s="462" t="n"/>
-      <c r="AF8" s="462" t="n"/>
-      <c r="AG8" s="462" t="n"/>
-      <c r="AH8" s="462" t="n"/>
-      <c r="AI8" s="462" t="n"/>
-      <c r="AJ8" s="462" t="n"/>
-      <c r="AK8" s="462" t="n"/>
-      <c r="AL8" s="462" t="n"/>
-      <c r="AM8" s="487" t="n"/>
-      <c r="AN8" s="488" t="n"/>
-      <c r="AO8" s="488" t="n"/>
-      <c r="AP8" s="488" t="n"/>
-      <c r="AQ8" s="488" t="n"/>
-      <c r="AR8" s="488" t="n"/>
-      <c r="AS8" s="488" t="n"/>
-      <c r="AT8" s="488" t="n"/>
-      <c r="AU8" s="488" t="n"/>
-      <c r="AV8" s="488" t="n"/>
-      <c r="AW8" s="488" t="n"/>
-      <c r="AX8" s="488" t="n"/>
-      <c r="AY8" s="488" t="n"/>
-      <c r="AZ8" s="488" t="n"/>
-      <c r="BA8" s="488" t="n"/>
-      <c r="BB8" s="488" t="n"/>
-      <c r="BC8" s="488" t="n"/>
-      <c r="BD8" s="489" t="n"/>
+      <c r="AD8" s="536" t="n"/>
+      <c r="AE8" s="536" t="n"/>
+      <c r="AF8" s="536" t="n"/>
+      <c r="AG8" s="536" t="n"/>
+      <c r="AH8" s="536" t="n"/>
+      <c r="AI8" s="536" t="n"/>
+      <c r="AJ8" s="536" t="n"/>
+      <c r="AK8" s="536" t="n"/>
+      <c r="AL8" s="536" t="n"/>
+      <c r="AM8" s="561" t="n"/>
+      <c r="AN8" s="560" t="n"/>
+      <c r="AO8" s="560" t="n"/>
+      <c r="AP8" s="560" t="n"/>
+      <c r="AQ8" s="560" t="n"/>
+      <c r="AR8" s="560" t="n"/>
+      <c r="AS8" s="560" t="n"/>
+      <c r="AT8" s="560" t="n"/>
+      <c r="AU8" s="560" t="n"/>
+      <c r="AV8" s="560" t="n"/>
+      <c r="AW8" s="560" t="n"/>
+      <c r="AX8" s="560" t="n"/>
+      <c r="AY8" s="560" t="n"/>
+      <c r="AZ8" s="560" t="n"/>
+      <c r="BA8" s="560" t="n"/>
+      <c r="BB8" s="560" t="n"/>
+      <c r="BC8" s="560" t="n"/>
+      <c r="BD8" s="562" t="n"/>
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="479" t="inlineStr">
@@ -8558,65 +8888,65 @@
           <t>Supplier / Processor</t>
         </is>
       </c>
-      <c r="B9" s="349" t="n"/>
-      <c r="C9" s="349" t="n"/>
-      <c r="D9" s="349" t="n"/>
-      <c r="E9" s="349" t="n"/>
-      <c r="F9" s="349" t="n"/>
-      <c r="G9" s="349" t="n"/>
-      <c r="H9" s="349" t="n"/>
-      <c r="I9" s="349" t="n"/>
-      <c r="J9" s="349" t="n"/>
+      <c r="B9" s="408" t="n"/>
+      <c r="C9" s="408" t="n"/>
+      <c r="D9" s="408" t="n"/>
+      <c r="E9" s="408" t="n"/>
+      <c r="F9" s="408" t="n"/>
+      <c r="G9" s="408" t="n"/>
+      <c r="H9" s="408" t="n"/>
+      <c r="I9" s="408" t="n"/>
+      <c r="J9" s="408" t="n"/>
       <c r="K9" s="490" t="n"/>
-      <c r="L9" s="380" t="n"/>
-      <c r="M9" s="380" t="n"/>
-      <c r="N9" s="380" t="n"/>
-      <c r="O9" s="380" t="n"/>
-      <c r="P9" s="380" t="n"/>
-      <c r="Q9" s="380" t="n"/>
-      <c r="R9" s="380" t="n"/>
-      <c r="S9" s="380" t="n"/>
-      <c r="T9" s="380" t="n"/>
-      <c r="U9" s="380" t="n"/>
-      <c r="V9" s="380" t="n"/>
-      <c r="W9" s="380" t="n"/>
-      <c r="X9" s="380" t="n"/>
-      <c r="Y9" s="380" t="n"/>
-      <c r="Z9" s="380" t="n"/>
-      <c r="AA9" s="380" t="n"/>
-      <c r="AB9" s="380" t="n"/>
+      <c r="L9" s="563" t="n"/>
+      <c r="M9" s="563" t="n"/>
+      <c r="N9" s="563" t="n"/>
+      <c r="O9" s="563" t="n"/>
+      <c r="P9" s="563" t="n"/>
+      <c r="Q9" s="563" t="n"/>
+      <c r="R9" s="563" t="n"/>
+      <c r="S9" s="563" t="n"/>
+      <c r="T9" s="563" t="n"/>
+      <c r="U9" s="563" t="n"/>
+      <c r="V9" s="563" t="n"/>
+      <c r="W9" s="563" t="n"/>
+      <c r="X9" s="563" t="n"/>
+      <c r="Y9" s="563" t="n"/>
+      <c r="Z9" s="563" t="n"/>
+      <c r="AA9" s="563" t="n"/>
+      <c r="AB9" s="563" t="n"/>
       <c r="AC9" s="481" t="inlineStr">
         <is>
           <t>Promise / Due Date</t>
         </is>
       </c>
-      <c r="AD9" s="349" t="n"/>
-      <c r="AE9" s="349" t="n"/>
-      <c r="AF9" s="349" t="n"/>
-      <c r="AG9" s="349" t="n"/>
-      <c r="AH9" s="349" t="n"/>
-      <c r="AI9" s="349" t="n"/>
-      <c r="AJ9" s="349" t="n"/>
-      <c r="AK9" s="349" t="n"/>
-      <c r="AL9" s="349" t="n"/>
-      <c r="AM9" s="490" t="n"/>
-      <c r="AN9" s="380" t="n"/>
-      <c r="AO9" s="380" t="n"/>
-      <c r="AP9" s="380" t="n"/>
-      <c r="AQ9" s="380" t="n"/>
-      <c r="AR9" s="380" t="n"/>
-      <c r="AS9" s="380" t="n"/>
-      <c r="AT9" s="380" t="n"/>
-      <c r="AU9" s="380" t="n"/>
-      <c r="AV9" s="380" t="n"/>
-      <c r="AW9" s="380" t="n"/>
-      <c r="AX9" s="380" t="n"/>
-      <c r="AY9" s="380" t="n"/>
-      <c r="AZ9" s="380" t="n"/>
-      <c r="BA9" s="380" t="n"/>
-      <c r="BB9" s="380" t="n"/>
-      <c r="BC9" s="380" t="n"/>
-      <c r="BD9" s="491" t="n"/>
+      <c r="AD9" s="408" t="n"/>
+      <c r="AE9" s="408" t="n"/>
+      <c r="AF9" s="408" t="n"/>
+      <c r="AG9" s="408" t="n"/>
+      <c r="AH9" s="408" t="n"/>
+      <c r="AI9" s="408" t="n"/>
+      <c r="AJ9" s="408" t="n"/>
+      <c r="AK9" s="408" t="n"/>
+      <c r="AL9" s="408" t="n"/>
+      <c r="AM9" s="564" t="n"/>
+      <c r="AN9" s="563" t="n"/>
+      <c r="AO9" s="563" t="n"/>
+      <c r="AP9" s="563" t="n"/>
+      <c r="AQ9" s="563" t="n"/>
+      <c r="AR9" s="563" t="n"/>
+      <c r="AS9" s="563" t="n"/>
+      <c r="AT9" s="563" t="n"/>
+      <c r="AU9" s="563" t="n"/>
+      <c r="AV9" s="563" t="n"/>
+      <c r="AW9" s="563" t="n"/>
+      <c r="AX9" s="563" t="n"/>
+      <c r="AY9" s="563" t="n"/>
+      <c r="AZ9" s="563" t="n"/>
+      <c r="BA9" s="563" t="n"/>
+      <c r="BB9" s="563" t="n"/>
+      <c r="BC9" s="563" t="n"/>
+      <c r="BD9" s="565" t="n"/>
     </row>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="479" t="inlineStr">
@@ -8624,65 +8954,65 @@
           <t>PO / Cert / Lot Ref</t>
         </is>
       </c>
-      <c r="B10" s="349" t="n"/>
-      <c r="C10" s="349" t="n"/>
-      <c r="D10" s="349" t="n"/>
-      <c r="E10" s="349" t="n"/>
-      <c r="F10" s="349" t="n"/>
-      <c r="G10" s="349" t="n"/>
-      <c r="H10" s="349" t="n"/>
-      <c r="I10" s="349" t="n"/>
-      <c r="J10" s="349" t="n"/>
+      <c r="B10" s="408" t="n"/>
+      <c r="C10" s="408" t="n"/>
+      <c r="D10" s="408" t="n"/>
+      <c r="E10" s="408" t="n"/>
+      <c r="F10" s="408" t="n"/>
+      <c r="G10" s="408" t="n"/>
+      <c r="H10" s="408" t="n"/>
+      <c r="I10" s="408" t="n"/>
+      <c r="J10" s="408" t="n"/>
       <c r="K10" s="490" t="n"/>
-      <c r="L10" s="380" t="n"/>
-      <c r="M10" s="380" t="n"/>
-      <c r="N10" s="380" t="n"/>
-      <c r="O10" s="380" t="n"/>
-      <c r="P10" s="380" t="n"/>
-      <c r="Q10" s="380" t="n"/>
-      <c r="R10" s="380" t="n"/>
-      <c r="S10" s="380" t="n"/>
-      <c r="T10" s="380" t="n"/>
-      <c r="U10" s="380" t="n"/>
-      <c r="V10" s="380" t="n"/>
-      <c r="W10" s="380" t="n"/>
-      <c r="X10" s="380" t="n"/>
-      <c r="Y10" s="380" t="n"/>
-      <c r="Z10" s="380" t="n"/>
-      <c r="AA10" s="380" t="n"/>
-      <c r="AB10" s="380" t="n"/>
+      <c r="L10" s="563" t="n"/>
+      <c r="M10" s="563" t="n"/>
+      <c r="N10" s="563" t="n"/>
+      <c r="O10" s="563" t="n"/>
+      <c r="P10" s="563" t="n"/>
+      <c r="Q10" s="563" t="n"/>
+      <c r="R10" s="563" t="n"/>
+      <c r="S10" s="563" t="n"/>
+      <c r="T10" s="563" t="n"/>
+      <c r="U10" s="563" t="n"/>
+      <c r="V10" s="563" t="n"/>
+      <c r="W10" s="563" t="n"/>
+      <c r="X10" s="563" t="n"/>
+      <c r="Y10" s="563" t="n"/>
+      <c r="Z10" s="563" t="n"/>
+      <c r="AA10" s="563" t="n"/>
+      <c r="AB10" s="563" t="n"/>
       <c r="AC10" s="481" t="inlineStr">
         <is>
           <t>Supplier-Quality Owner</t>
         </is>
       </c>
-      <c r="AD10" s="349" t="n"/>
-      <c r="AE10" s="349" t="n"/>
-      <c r="AF10" s="349" t="n"/>
-      <c r="AG10" s="349" t="n"/>
-      <c r="AH10" s="349" t="n"/>
-      <c r="AI10" s="349" t="n"/>
-      <c r="AJ10" s="349" t="n"/>
-      <c r="AK10" s="349" t="n"/>
-      <c r="AL10" s="349" t="n"/>
-      <c r="AM10" s="490" t="n"/>
-      <c r="AN10" s="380" t="n"/>
-      <c r="AO10" s="380" t="n"/>
-      <c r="AP10" s="380" t="n"/>
-      <c r="AQ10" s="380" t="n"/>
-      <c r="AR10" s="380" t="n"/>
-      <c r="AS10" s="380" t="n"/>
-      <c r="AT10" s="380" t="n"/>
-      <c r="AU10" s="380" t="n"/>
-      <c r="AV10" s="380" t="n"/>
-      <c r="AW10" s="380" t="n"/>
-      <c r="AX10" s="380" t="n"/>
-      <c r="AY10" s="380" t="n"/>
-      <c r="AZ10" s="380" t="n"/>
-      <c r="BA10" s="380" t="n"/>
-      <c r="BB10" s="380" t="n"/>
-      <c r="BC10" s="380" t="n"/>
-      <c r="BD10" s="491" t="n"/>
+      <c r="AD10" s="408" t="n"/>
+      <c r="AE10" s="408" t="n"/>
+      <c r="AF10" s="408" t="n"/>
+      <c r="AG10" s="408" t="n"/>
+      <c r="AH10" s="408" t="n"/>
+      <c r="AI10" s="408" t="n"/>
+      <c r="AJ10" s="408" t="n"/>
+      <c r="AK10" s="408" t="n"/>
+      <c r="AL10" s="408" t="n"/>
+      <c r="AM10" s="564" t="n"/>
+      <c r="AN10" s="563" t="n"/>
+      <c r="AO10" s="563" t="n"/>
+      <c r="AP10" s="563" t="n"/>
+      <c r="AQ10" s="563" t="n"/>
+      <c r="AR10" s="563" t="n"/>
+      <c r="AS10" s="563" t="n"/>
+      <c r="AT10" s="563" t="n"/>
+      <c r="AU10" s="563" t="n"/>
+      <c r="AV10" s="563" t="n"/>
+      <c r="AW10" s="563" t="n"/>
+      <c r="AX10" s="563" t="n"/>
+      <c r="AY10" s="563" t="n"/>
+      <c r="AZ10" s="563" t="n"/>
+      <c r="BA10" s="563" t="n"/>
+      <c r="BB10" s="563" t="n"/>
+      <c r="BC10" s="563" t="n"/>
+      <c r="BD10" s="565" t="n"/>
     </row>
     <row r="11" ht="26" customHeight="1">
       <c r="A11" s="492" t="inlineStr">
@@ -8690,65 +9020,65 @@
           <t>Prepared by / Date-Time</t>
         </is>
       </c>
-      <c r="B11" s="493" t="n"/>
-      <c r="C11" s="493" t="n"/>
-      <c r="D11" s="493" t="n"/>
-      <c r="E11" s="493" t="n"/>
-      <c r="F11" s="493" t="n"/>
-      <c r="G11" s="493" t="n"/>
-      <c r="H11" s="493" t="n"/>
-      <c r="I11" s="493" t="n"/>
-      <c r="J11" s="493" t="n"/>
+      <c r="B11" s="554" t="n"/>
+      <c r="C11" s="554" t="n"/>
+      <c r="D11" s="554" t="n"/>
+      <c r="E11" s="554" t="n"/>
+      <c r="F11" s="554" t="n"/>
+      <c r="G11" s="554" t="n"/>
+      <c r="H11" s="554" t="n"/>
+      <c r="I11" s="554" t="n"/>
+      <c r="J11" s="554" t="n"/>
       <c r="K11" s="494" t="n"/>
-      <c r="L11" s="495" t="n"/>
-      <c r="M11" s="495" t="n"/>
-      <c r="N11" s="495" t="n"/>
-      <c r="O11" s="495" t="n"/>
-      <c r="P11" s="495" t="n"/>
-      <c r="Q11" s="495" t="n"/>
-      <c r="R11" s="495" t="n"/>
-      <c r="S11" s="495" t="n"/>
-      <c r="T11" s="495" t="n"/>
-      <c r="U11" s="495" t="n"/>
-      <c r="V11" s="495" t="n"/>
-      <c r="W11" s="495" t="n"/>
-      <c r="X11" s="495" t="n"/>
-      <c r="Y11" s="495" t="n"/>
-      <c r="Z11" s="495" t="n"/>
-      <c r="AA11" s="495" t="n"/>
-      <c r="AB11" s="495" t="n"/>
+      <c r="L11" s="566" t="n"/>
+      <c r="M11" s="566" t="n"/>
+      <c r="N11" s="566" t="n"/>
+      <c r="O11" s="566" t="n"/>
+      <c r="P11" s="566" t="n"/>
+      <c r="Q11" s="566" t="n"/>
+      <c r="R11" s="566" t="n"/>
+      <c r="S11" s="566" t="n"/>
+      <c r="T11" s="566" t="n"/>
+      <c r="U11" s="566" t="n"/>
+      <c r="V11" s="566" t="n"/>
+      <c r="W11" s="566" t="n"/>
+      <c r="X11" s="566" t="n"/>
+      <c r="Y11" s="566" t="n"/>
+      <c r="Z11" s="566" t="n"/>
+      <c r="AA11" s="566" t="n"/>
+      <c r="AB11" s="566" t="n"/>
       <c r="AC11" s="496" t="inlineStr">
         <is>
           <t>Evidence Package Ref</t>
         </is>
       </c>
-      <c r="AD11" s="493" t="n"/>
-      <c r="AE11" s="493" t="n"/>
-      <c r="AF11" s="493" t="n"/>
-      <c r="AG11" s="493" t="n"/>
-      <c r="AH11" s="493" t="n"/>
-      <c r="AI11" s="493" t="n"/>
-      <c r="AJ11" s="493" t="n"/>
-      <c r="AK11" s="493" t="n"/>
-      <c r="AL11" s="493" t="n"/>
-      <c r="AM11" s="494" t="n"/>
-      <c r="AN11" s="495" t="n"/>
-      <c r="AO11" s="495" t="n"/>
-      <c r="AP11" s="495" t="n"/>
-      <c r="AQ11" s="495" t="n"/>
-      <c r="AR11" s="495" t="n"/>
-      <c r="AS11" s="495" t="n"/>
-      <c r="AT11" s="495" t="n"/>
-      <c r="AU11" s="495" t="n"/>
-      <c r="AV11" s="495" t="n"/>
-      <c r="AW11" s="495" t="n"/>
-      <c r="AX11" s="495" t="n"/>
-      <c r="AY11" s="495" t="n"/>
-      <c r="AZ11" s="495" t="n"/>
-      <c r="BA11" s="495" t="n"/>
-      <c r="BB11" s="495" t="n"/>
-      <c r="BC11" s="495" t="n"/>
-      <c r="BD11" s="497" t="n"/>
+      <c r="AD11" s="554" t="n"/>
+      <c r="AE11" s="554" t="n"/>
+      <c r="AF11" s="554" t="n"/>
+      <c r="AG11" s="554" t="n"/>
+      <c r="AH11" s="554" t="n"/>
+      <c r="AI11" s="554" t="n"/>
+      <c r="AJ11" s="554" t="n"/>
+      <c r="AK11" s="554" t="n"/>
+      <c r="AL11" s="554" t="n"/>
+      <c r="AM11" s="567" t="n"/>
+      <c r="AN11" s="566" t="n"/>
+      <c r="AO11" s="566" t="n"/>
+      <c r="AP11" s="566" t="n"/>
+      <c r="AQ11" s="566" t="n"/>
+      <c r="AR11" s="566" t="n"/>
+      <c r="AS11" s="566" t="n"/>
+      <c r="AT11" s="566" t="n"/>
+      <c r="AU11" s="566" t="n"/>
+      <c r="AV11" s="566" t="n"/>
+      <c r="AW11" s="566" t="n"/>
+      <c r="AX11" s="566" t="n"/>
+      <c r="AY11" s="566" t="n"/>
+      <c r="AZ11" s="566" t="n"/>
+      <c r="BA11" s="566" t="n"/>
+      <c r="BB11" s="566" t="n"/>
+      <c r="BC11" s="566" t="n"/>
+      <c r="BD11" s="568" t="n"/>
     </row>
     <row r="12" ht="3" customHeight="1">
       <c r="A12" s="382" t="n"/>
@@ -8809,66 +9139,66 @@
       <c r="BD12" s="354" t="n"/>
     </row>
     <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="472" t="inlineStr">
+      <c r="A13" s="558" t="inlineStr">
         <is>
           <t xml:space="preserve">  2. REVIEW SNAPSHOT / LIVE ENTRY ON PO_DATA_LOG</t>
         </is>
       </c>
-      <c r="B13" s="473" t="n"/>
-      <c r="C13" s="473" t="n"/>
-      <c r="D13" s="473" t="n"/>
-      <c r="E13" s="473" t="n"/>
-      <c r="F13" s="473" t="n"/>
-      <c r="G13" s="473" t="n"/>
-      <c r="H13" s="473" t="n"/>
-      <c r="I13" s="473" t="n"/>
-      <c r="J13" s="473" t="n"/>
-      <c r="K13" s="473" t="n"/>
-      <c r="L13" s="473" t="n"/>
-      <c r="M13" s="473" t="n"/>
-      <c r="N13" s="473" t="n"/>
-      <c r="O13" s="473" t="n"/>
-      <c r="P13" s="473" t="n"/>
-      <c r="Q13" s="473" t="n"/>
-      <c r="R13" s="473" t="n"/>
-      <c r="S13" s="473" t="n"/>
-      <c r="T13" s="473" t="n"/>
-      <c r="U13" s="473" t="n"/>
-      <c r="V13" s="473" t="n"/>
-      <c r="W13" s="473" t="n"/>
-      <c r="X13" s="473" t="n"/>
-      <c r="Y13" s="473" t="n"/>
-      <c r="Z13" s="473" t="n"/>
-      <c r="AA13" s="473" t="n"/>
-      <c r="AB13" s="473" t="n"/>
-      <c r="AC13" s="473" t="n"/>
-      <c r="AD13" s="473" t="n"/>
-      <c r="AE13" s="473" t="n"/>
-      <c r="AF13" s="473" t="n"/>
-      <c r="AG13" s="473" t="n"/>
-      <c r="AH13" s="473" t="n"/>
-      <c r="AI13" s="473" t="n"/>
-      <c r="AJ13" s="473" t="n"/>
-      <c r="AK13" s="473" t="n"/>
-      <c r="AL13" s="473" t="n"/>
-      <c r="AM13" s="473" t="n"/>
-      <c r="AN13" s="473" t="n"/>
-      <c r="AO13" s="473" t="n"/>
-      <c r="AP13" s="473" t="n"/>
-      <c r="AQ13" s="473" t="n"/>
-      <c r="AR13" s="473" t="n"/>
-      <c r="AS13" s="473" t="n"/>
-      <c r="AT13" s="473" t="n"/>
-      <c r="AU13" s="473" t="n"/>
-      <c r="AV13" s="473" t="n"/>
-      <c r="AW13" s="473" t="n"/>
-      <c r="AX13" s="473" t="n"/>
-      <c r="AY13" s="473" t="n"/>
-      <c r="AZ13" s="473" t="n"/>
-      <c r="BA13" s="473" t="n"/>
-      <c r="BB13" s="473" t="n"/>
-      <c r="BC13" s="473" t="n"/>
-      <c r="BD13" s="474" t="n"/>
+      <c r="B13" s="535" t="n"/>
+      <c r="C13" s="535" t="n"/>
+      <c r="D13" s="535" t="n"/>
+      <c r="E13" s="535" t="n"/>
+      <c r="F13" s="535" t="n"/>
+      <c r="G13" s="535" t="n"/>
+      <c r="H13" s="535" t="n"/>
+      <c r="I13" s="535" t="n"/>
+      <c r="J13" s="535" t="n"/>
+      <c r="K13" s="535" t="n"/>
+      <c r="L13" s="535" t="n"/>
+      <c r="M13" s="535" t="n"/>
+      <c r="N13" s="535" t="n"/>
+      <c r="O13" s="535" t="n"/>
+      <c r="P13" s="535" t="n"/>
+      <c r="Q13" s="535" t="n"/>
+      <c r="R13" s="535" t="n"/>
+      <c r="S13" s="535" t="n"/>
+      <c r="T13" s="535" t="n"/>
+      <c r="U13" s="535" t="n"/>
+      <c r="V13" s="535" t="n"/>
+      <c r="W13" s="535" t="n"/>
+      <c r="X13" s="535" t="n"/>
+      <c r="Y13" s="535" t="n"/>
+      <c r="Z13" s="535" t="n"/>
+      <c r="AA13" s="535" t="n"/>
+      <c r="AB13" s="535" t="n"/>
+      <c r="AC13" s="535" t="n"/>
+      <c r="AD13" s="535" t="n"/>
+      <c r="AE13" s="535" t="n"/>
+      <c r="AF13" s="535" t="n"/>
+      <c r="AG13" s="535" t="n"/>
+      <c r="AH13" s="535" t="n"/>
+      <c r="AI13" s="535" t="n"/>
+      <c r="AJ13" s="535" t="n"/>
+      <c r="AK13" s="535" t="n"/>
+      <c r="AL13" s="535" t="n"/>
+      <c r="AM13" s="535" t="n"/>
+      <c r="AN13" s="535" t="n"/>
+      <c r="AO13" s="535" t="n"/>
+      <c r="AP13" s="535" t="n"/>
+      <c r="AQ13" s="535" t="n"/>
+      <c r="AR13" s="535" t="n"/>
+      <c r="AS13" s="535" t="n"/>
+      <c r="AT13" s="535" t="n"/>
+      <c r="AU13" s="535" t="n"/>
+      <c r="AV13" s="535" t="n"/>
+      <c r="AW13" s="535" t="n"/>
+      <c r="AX13" s="535" t="n"/>
+      <c r="AY13" s="535" t="n"/>
+      <c r="AZ13" s="535" t="n"/>
+      <c r="BA13" s="535" t="n"/>
+      <c r="BB13" s="535" t="n"/>
+      <c r="BC13" s="535" t="n"/>
+      <c r="BD13" s="559" t="n"/>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="456" t="inlineStr">
@@ -8876,793 +9206,793 @@
           <t>#</t>
         </is>
       </c>
-      <c r="B14" s="457" t="n"/>
+      <c r="B14" s="535" t="n"/>
       <c r="C14" s="498" t="inlineStr">
         <is>
           <t>Date-Time</t>
         </is>
       </c>
-      <c r="D14" s="457" t="n"/>
-      <c r="E14" s="457" t="n"/>
-      <c r="F14" s="457" t="n"/>
-      <c r="G14" s="457" t="n"/>
+      <c r="D14" s="535" t="n"/>
+      <c r="E14" s="535" t="n"/>
+      <c r="F14" s="535" t="n"/>
+      <c r="G14" s="535" t="n"/>
       <c r="H14" s="498" t="inlineStr">
         <is>
           <t>PO / Promise Ref</t>
         </is>
       </c>
-      <c r="I14" s="457" t="n"/>
-      <c r="J14" s="457" t="n"/>
-      <c r="K14" s="457" t="n"/>
-      <c r="L14" s="457" t="n"/>
+      <c r="I14" s="535" t="n"/>
+      <c r="J14" s="535" t="n"/>
+      <c r="K14" s="535" t="n"/>
+      <c r="L14" s="535" t="n"/>
       <c r="M14" s="498" t="inlineStr">
         <is>
           <t>Supplier / Processor</t>
         </is>
       </c>
-      <c r="N14" s="457" t="n"/>
-      <c r="O14" s="457" t="n"/>
-      <c r="P14" s="457" t="n"/>
-      <c r="Q14" s="457" t="n"/>
+      <c r="N14" s="535" t="n"/>
+      <c r="O14" s="535" t="n"/>
+      <c r="P14" s="535" t="n"/>
+      <c r="Q14" s="535" t="n"/>
       <c r="R14" s="498" t="inlineStr">
         <is>
           <t>Issue / Exception</t>
         </is>
       </c>
-      <c r="S14" s="457" t="n"/>
-      <c r="T14" s="457" t="n"/>
-      <c r="U14" s="457" t="n"/>
-      <c r="V14" s="457" t="n"/>
+      <c r="S14" s="535" t="n"/>
+      <c r="T14" s="535" t="n"/>
+      <c r="U14" s="535" t="n"/>
+      <c r="V14" s="535" t="n"/>
       <c r="W14" s="498" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="X14" s="457" t="n"/>
-      <c r="Y14" s="457" t="n"/>
-      <c r="Z14" s="457" t="n"/>
+      <c r="X14" s="535" t="n"/>
+      <c r="Y14" s="535" t="n"/>
+      <c r="Z14" s="535" t="n"/>
       <c r="AA14" s="498" t="inlineStr">
         <is>
           <t>Risk</t>
         </is>
       </c>
-      <c r="AB14" s="457" t="n"/>
-      <c r="AC14" s="457" t="n"/>
-      <c r="AD14" s="457" t="n"/>
+      <c r="AB14" s="535" t="n"/>
+      <c r="AC14" s="535" t="n"/>
+      <c r="AD14" s="535" t="n"/>
       <c r="AE14" s="498" t="inlineStr">
         <is>
           <t>Owner Dept</t>
         </is>
       </c>
-      <c r="AF14" s="457" t="n"/>
-      <c r="AG14" s="457" t="n"/>
-      <c r="AH14" s="457" t="n"/>
+      <c r="AF14" s="535" t="n"/>
+      <c r="AG14" s="535" t="n"/>
+      <c r="AH14" s="535" t="n"/>
       <c r="AI14" s="498" t="inlineStr">
         <is>
           <t>Required Action</t>
         </is>
       </c>
-      <c r="AJ14" s="457" t="n"/>
-      <c r="AK14" s="457" t="n"/>
-      <c r="AL14" s="457" t="n"/>
-      <c r="AM14" s="457" t="n"/>
+      <c r="AJ14" s="535" t="n"/>
+      <c r="AK14" s="535" t="n"/>
+      <c r="AL14" s="535" t="n"/>
+      <c r="AM14" s="535" t="n"/>
       <c r="AN14" s="498" t="inlineStr">
         <is>
           <t>Evidence Ref</t>
         </is>
       </c>
-      <c r="AO14" s="457" t="n"/>
-      <c r="AP14" s="457" t="n"/>
-      <c r="AQ14" s="457" t="n"/>
+      <c r="AO14" s="535" t="n"/>
+      <c r="AP14" s="535" t="n"/>
+      <c r="AQ14" s="535" t="n"/>
       <c r="AR14" s="498" t="n"/>
-      <c r="AS14" s="457" t="n"/>
-      <c r="AT14" s="457" t="n"/>
-      <c r="AU14" s="457" t="n"/>
+      <c r="AS14" s="535" t="n"/>
+      <c r="AT14" s="535" t="n"/>
+      <c r="AU14" s="535" t="n"/>
       <c r="AV14" s="498" t="n"/>
-      <c r="AW14" s="457" t="n"/>
-      <c r="AX14" s="457" t="n"/>
-      <c r="AY14" s="457" t="n"/>
-      <c r="AZ14" s="498" t="n"/>
-      <c r="BA14" s="457" t="n"/>
-      <c r="BB14" s="457" t="n"/>
-      <c r="BC14" s="457" t="n"/>
-      <c r="BD14" s="458" t="n"/>
+      <c r="AW14" s="535" t="n"/>
+      <c r="AX14" s="535" t="n"/>
+      <c r="AY14" s="535" t="n"/>
+      <c r="AZ14" s="569" t="n"/>
+      <c r="BA14" s="535" t="n"/>
+      <c r="BB14" s="535" t="n"/>
+      <c r="BC14" s="535" t="n"/>
+      <c r="BD14" s="559" t="n"/>
     </row>
     <row r="15" ht="20" customHeight="1">
       <c r="A15" s="499" t="n"/>
-      <c r="B15" s="462" t="n"/>
+      <c r="B15" s="536" t="n"/>
       <c r="C15" s="500" t="n"/>
-      <c r="D15" s="488" t="n"/>
-      <c r="E15" s="488" t="n"/>
-      <c r="F15" s="488" t="n"/>
-      <c r="G15" s="488" t="n"/>
+      <c r="D15" s="560" t="n"/>
+      <c r="E15" s="560" t="n"/>
+      <c r="F15" s="560" t="n"/>
+      <c r="G15" s="560" t="n"/>
       <c r="H15" s="500" t="n"/>
-      <c r="I15" s="488" t="n"/>
-      <c r="J15" s="488" t="n"/>
-      <c r="K15" s="488" t="n"/>
-      <c r="L15" s="488" t="n"/>
+      <c r="I15" s="560" t="n"/>
+      <c r="J15" s="560" t="n"/>
+      <c r="K15" s="560" t="n"/>
+      <c r="L15" s="560" t="n"/>
       <c r="M15" s="500" t="n"/>
-      <c r="N15" s="488" t="n"/>
-      <c r="O15" s="488" t="n"/>
-      <c r="P15" s="488" t="n"/>
-      <c r="Q15" s="488" t="n"/>
+      <c r="N15" s="560" t="n"/>
+      <c r="O15" s="560" t="n"/>
+      <c r="P15" s="560" t="n"/>
+      <c r="Q15" s="560" t="n"/>
       <c r="R15" s="500" t="n"/>
-      <c r="S15" s="488" t="n"/>
-      <c r="T15" s="488" t="n"/>
-      <c r="U15" s="488" t="n"/>
-      <c r="V15" s="488" t="n"/>
+      <c r="S15" s="560" t="n"/>
+      <c r="T15" s="560" t="n"/>
+      <c r="U15" s="560" t="n"/>
+      <c r="V15" s="560" t="n"/>
       <c r="W15" s="500" t="n"/>
-      <c r="X15" s="488" t="n"/>
-      <c r="Y15" s="488" t="n"/>
-      <c r="Z15" s="488" t="n"/>
+      <c r="X15" s="560" t="n"/>
+      <c r="Y15" s="560" t="n"/>
+      <c r="Z15" s="560" t="n"/>
       <c r="AA15" s="500" t="n"/>
-      <c r="AB15" s="488" t="n"/>
-      <c r="AC15" s="488" t="n"/>
-      <c r="AD15" s="488" t="n"/>
+      <c r="AB15" s="560" t="n"/>
+      <c r="AC15" s="560" t="n"/>
+      <c r="AD15" s="560" t="n"/>
       <c r="AE15" s="500" t="n"/>
-      <c r="AF15" s="488" t="n"/>
-      <c r="AG15" s="488" t="n"/>
-      <c r="AH15" s="488" t="n"/>
+      <c r="AF15" s="560" t="n"/>
+      <c r="AG15" s="560" t="n"/>
+      <c r="AH15" s="560" t="n"/>
       <c r="AI15" s="500" t="n"/>
-      <c r="AJ15" s="488" t="n"/>
-      <c r="AK15" s="488" t="n"/>
-      <c r="AL15" s="488" t="n"/>
-      <c r="AM15" s="488" t="n"/>
+      <c r="AJ15" s="560" t="n"/>
+      <c r="AK15" s="560" t="n"/>
+      <c r="AL15" s="560" t="n"/>
+      <c r="AM15" s="560" t="n"/>
       <c r="AN15" s="500" t="n"/>
-      <c r="AO15" s="488" t="n"/>
-      <c r="AP15" s="488" t="n"/>
-      <c r="AQ15" s="488" t="n"/>
+      <c r="AO15" s="560" t="n"/>
+      <c r="AP15" s="560" t="n"/>
+      <c r="AQ15" s="560" t="n"/>
       <c r="AR15" s="500" t="n"/>
-      <c r="AS15" s="488" t="n"/>
-      <c r="AT15" s="488" t="n"/>
-      <c r="AU15" s="488" t="n"/>
+      <c r="AS15" s="560" t="n"/>
+      <c r="AT15" s="560" t="n"/>
+      <c r="AU15" s="560" t="n"/>
       <c r="AV15" s="500" t="n"/>
-      <c r="AW15" s="488" t="n"/>
-      <c r="AX15" s="488" t="n"/>
-      <c r="AY15" s="488" t="n"/>
-      <c r="AZ15" s="500" t="n"/>
-      <c r="BA15" s="488" t="n"/>
-      <c r="BB15" s="488" t="n"/>
-      <c r="BC15" s="488" t="n"/>
-      <c r="BD15" s="489" t="n"/>
+      <c r="AW15" s="560" t="n"/>
+      <c r="AX15" s="560" t="n"/>
+      <c r="AY15" s="560" t="n"/>
+      <c r="AZ15" s="570" t="n"/>
+      <c r="BA15" s="560" t="n"/>
+      <c r="BB15" s="560" t="n"/>
+      <c r="BC15" s="560" t="n"/>
+      <c r="BD15" s="562" t="n"/>
     </row>
     <row r="16" ht="20" customHeight="1">
       <c r="A16" s="501" t="n"/>
-      <c r="B16" s="349" t="n"/>
+      <c r="B16" s="408" t="n"/>
       <c r="C16" s="502" t="n"/>
-      <c r="D16" s="380" t="n"/>
-      <c r="E16" s="380" t="n"/>
-      <c r="F16" s="380" t="n"/>
-      <c r="G16" s="380" t="n"/>
+      <c r="D16" s="563" t="n"/>
+      <c r="E16" s="563" t="n"/>
+      <c r="F16" s="563" t="n"/>
+      <c r="G16" s="563" t="n"/>
       <c r="H16" s="502" t="n"/>
-      <c r="I16" s="380" t="n"/>
-      <c r="J16" s="380" t="n"/>
-      <c r="K16" s="380" t="n"/>
-      <c r="L16" s="380" t="n"/>
+      <c r="I16" s="563" t="n"/>
+      <c r="J16" s="563" t="n"/>
+      <c r="K16" s="563" t="n"/>
+      <c r="L16" s="563" t="n"/>
       <c r="M16" s="502" t="n"/>
-      <c r="N16" s="380" t="n"/>
-      <c r="O16" s="380" t="n"/>
-      <c r="P16" s="380" t="n"/>
-      <c r="Q16" s="380" t="n"/>
+      <c r="N16" s="563" t="n"/>
+      <c r="O16" s="563" t="n"/>
+      <c r="P16" s="563" t="n"/>
+      <c r="Q16" s="563" t="n"/>
       <c r="R16" s="502" t="n"/>
-      <c r="S16" s="380" t="n"/>
-      <c r="T16" s="380" t="n"/>
-      <c r="U16" s="380" t="n"/>
-      <c r="V16" s="380" t="n"/>
+      <c r="S16" s="563" t="n"/>
+      <c r="T16" s="563" t="n"/>
+      <c r="U16" s="563" t="n"/>
+      <c r="V16" s="563" t="n"/>
       <c r="W16" s="502" t="n"/>
-      <c r="X16" s="380" t="n"/>
-      <c r="Y16" s="380" t="n"/>
-      <c r="Z16" s="380" t="n"/>
+      <c r="X16" s="563" t="n"/>
+      <c r="Y16" s="563" t="n"/>
+      <c r="Z16" s="563" t="n"/>
       <c r="AA16" s="502" t="n"/>
-      <c r="AB16" s="380" t="n"/>
-      <c r="AC16" s="380" t="n"/>
-      <c r="AD16" s="380" t="n"/>
+      <c r="AB16" s="563" t="n"/>
+      <c r="AC16" s="563" t="n"/>
+      <c r="AD16" s="563" t="n"/>
       <c r="AE16" s="502" t="n"/>
-      <c r="AF16" s="380" t="n"/>
-      <c r="AG16" s="380" t="n"/>
-      <c r="AH16" s="380" t="n"/>
+      <c r="AF16" s="563" t="n"/>
+      <c r="AG16" s="563" t="n"/>
+      <c r="AH16" s="563" t="n"/>
       <c r="AI16" s="502" t="n"/>
-      <c r="AJ16" s="380" t="n"/>
-      <c r="AK16" s="380" t="n"/>
-      <c r="AL16" s="380" t="n"/>
-      <c r="AM16" s="380" t="n"/>
+      <c r="AJ16" s="563" t="n"/>
+      <c r="AK16" s="563" t="n"/>
+      <c r="AL16" s="563" t="n"/>
+      <c r="AM16" s="563" t="n"/>
       <c r="AN16" s="502" t="n"/>
-      <c r="AO16" s="380" t="n"/>
-      <c r="AP16" s="380" t="n"/>
-      <c r="AQ16" s="380" t="n"/>
+      <c r="AO16" s="563" t="n"/>
+      <c r="AP16" s="563" t="n"/>
+      <c r="AQ16" s="563" t="n"/>
       <c r="AR16" s="502" t="n"/>
-      <c r="AS16" s="380" t="n"/>
-      <c r="AT16" s="380" t="n"/>
-      <c r="AU16" s="380" t="n"/>
+      <c r="AS16" s="563" t="n"/>
+      <c r="AT16" s="563" t="n"/>
+      <c r="AU16" s="563" t="n"/>
       <c r="AV16" s="502" t="n"/>
-      <c r="AW16" s="380" t="n"/>
-      <c r="AX16" s="380" t="n"/>
-      <c r="AY16" s="380" t="n"/>
-      <c r="AZ16" s="502" t="n"/>
-      <c r="BA16" s="380" t="n"/>
-      <c r="BB16" s="380" t="n"/>
-      <c r="BC16" s="380" t="n"/>
-      <c r="BD16" s="491" t="n"/>
+      <c r="AW16" s="563" t="n"/>
+      <c r="AX16" s="563" t="n"/>
+      <c r="AY16" s="563" t="n"/>
+      <c r="AZ16" s="571" t="n"/>
+      <c r="BA16" s="563" t="n"/>
+      <c r="BB16" s="563" t="n"/>
+      <c r="BC16" s="563" t="n"/>
+      <c r="BD16" s="565" t="n"/>
     </row>
     <row r="17" ht="20" customHeight="1">
       <c r="A17" s="501" t="n"/>
-      <c r="B17" s="349" t="n"/>
+      <c r="B17" s="408" t="n"/>
       <c r="C17" s="502" t="n"/>
-      <c r="D17" s="380" t="n"/>
-      <c r="E17" s="380" t="n"/>
-      <c r="F17" s="380" t="n"/>
-      <c r="G17" s="380" t="n"/>
+      <c r="D17" s="563" t="n"/>
+      <c r="E17" s="563" t="n"/>
+      <c r="F17" s="563" t="n"/>
+      <c r="G17" s="563" t="n"/>
       <c r="H17" s="502" t="n"/>
-      <c r="I17" s="380" t="n"/>
-      <c r="J17" s="380" t="n"/>
-      <c r="K17" s="380" t="n"/>
-      <c r="L17" s="380" t="n"/>
+      <c r="I17" s="563" t="n"/>
+      <c r="J17" s="563" t="n"/>
+      <c r="K17" s="563" t="n"/>
+      <c r="L17" s="563" t="n"/>
       <c r="M17" s="502" t="n"/>
-      <c r="N17" s="380" t="n"/>
-      <c r="O17" s="380" t="n"/>
-      <c r="P17" s="380" t="n"/>
-      <c r="Q17" s="380" t="n"/>
+      <c r="N17" s="563" t="n"/>
+      <c r="O17" s="563" t="n"/>
+      <c r="P17" s="563" t="n"/>
+      <c r="Q17" s="563" t="n"/>
       <c r="R17" s="502" t="n"/>
-      <c r="S17" s="380" t="n"/>
-      <c r="T17" s="380" t="n"/>
-      <c r="U17" s="380" t="n"/>
-      <c r="V17" s="380" t="n"/>
+      <c r="S17" s="563" t="n"/>
+      <c r="T17" s="563" t="n"/>
+      <c r="U17" s="563" t="n"/>
+      <c r="V17" s="563" t="n"/>
       <c r="W17" s="502" t="n"/>
-      <c r="X17" s="380" t="n"/>
-      <c r="Y17" s="380" t="n"/>
-      <c r="Z17" s="380" t="n"/>
+      <c r="X17" s="563" t="n"/>
+      <c r="Y17" s="563" t="n"/>
+      <c r="Z17" s="563" t="n"/>
       <c r="AA17" s="502" t="n"/>
-      <c r="AB17" s="380" t="n"/>
-      <c r="AC17" s="380" t="n"/>
-      <c r="AD17" s="380" t="n"/>
+      <c r="AB17" s="563" t="n"/>
+      <c r="AC17" s="563" t="n"/>
+      <c r="AD17" s="563" t="n"/>
       <c r="AE17" s="502" t="n"/>
-      <c r="AF17" s="380" t="n"/>
-      <c r="AG17" s="380" t="n"/>
-      <c r="AH17" s="380" t="n"/>
+      <c r="AF17" s="563" t="n"/>
+      <c r="AG17" s="563" t="n"/>
+      <c r="AH17" s="563" t="n"/>
       <c r="AI17" s="502" t="n"/>
-      <c r="AJ17" s="380" t="n"/>
-      <c r="AK17" s="380" t="n"/>
-      <c r="AL17" s="380" t="n"/>
-      <c r="AM17" s="380" t="n"/>
+      <c r="AJ17" s="563" t="n"/>
+      <c r="AK17" s="563" t="n"/>
+      <c r="AL17" s="563" t="n"/>
+      <c r="AM17" s="563" t="n"/>
       <c r="AN17" s="502" t="n"/>
-      <c r="AO17" s="380" t="n"/>
-      <c r="AP17" s="380" t="n"/>
-      <c r="AQ17" s="380" t="n"/>
+      <c r="AO17" s="563" t="n"/>
+      <c r="AP17" s="563" t="n"/>
+      <c r="AQ17" s="563" t="n"/>
       <c r="AR17" s="502" t="n"/>
-      <c r="AS17" s="380" t="n"/>
-      <c r="AT17" s="380" t="n"/>
-      <c r="AU17" s="380" t="n"/>
+      <c r="AS17" s="563" t="n"/>
+      <c r="AT17" s="563" t="n"/>
+      <c r="AU17" s="563" t="n"/>
       <c r="AV17" s="502" t="n"/>
-      <c r="AW17" s="380" t="n"/>
-      <c r="AX17" s="380" t="n"/>
-      <c r="AY17" s="380" t="n"/>
-      <c r="AZ17" s="502" t="n"/>
-      <c r="BA17" s="380" t="n"/>
-      <c r="BB17" s="380" t="n"/>
-      <c r="BC17" s="380" t="n"/>
-      <c r="BD17" s="491" t="n"/>
+      <c r="AW17" s="563" t="n"/>
+      <c r="AX17" s="563" t="n"/>
+      <c r="AY17" s="563" t="n"/>
+      <c r="AZ17" s="571" t="n"/>
+      <c r="BA17" s="563" t="n"/>
+      <c r="BB17" s="563" t="n"/>
+      <c r="BC17" s="563" t="n"/>
+      <c r="BD17" s="565" t="n"/>
     </row>
     <row r="18" ht="20" customHeight="1">
       <c r="A18" s="501" t="n"/>
-      <c r="B18" s="349" t="n"/>
+      <c r="B18" s="408" t="n"/>
       <c r="C18" s="502" t="n"/>
-      <c r="D18" s="380" t="n"/>
-      <c r="E18" s="380" t="n"/>
-      <c r="F18" s="380" t="n"/>
-      <c r="G18" s="380" t="n"/>
+      <c r="D18" s="563" t="n"/>
+      <c r="E18" s="563" t="n"/>
+      <c r="F18" s="563" t="n"/>
+      <c r="G18" s="563" t="n"/>
       <c r="H18" s="502" t="n"/>
-      <c r="I18" s="380" t="n"/>
-      <c r="J18" s="380" t="n"/>
-      <c r="K18" s="380" t="n"/>
-      <c r="L18" s="380" t="n"/>
+      <c r="I18" s="563" t="n"/>
+      <c r="J18" s="563" t="n"/>
+      <c r="K18" s="563" t="n"/>
+      <c r="L18" s="563" t="n"/>
       <c r="M18" s="502" t="n"/>
-      <c r="N18" s="380" t="n"/>
-      <c r="O18" s="380" t="n"/>
-      <c r="P18" s="380" t="n"/>
-      <c r="Q18" s="380" t="n"/>
+      <c r="N18" s="563" t="n"/>
+      <c r="O18" s="563" t="n"/>
+      <c r="P18" s="563" t="n"/>
+      <c r="Q18" s="563" t="n"/>
       <c r="R18" s="502" t="n"/>
-      <c r="S18" s="380" t="n"/>
-      <c r="T18" s="380" t="n"/>
-      <c r="U18" s="380" t="n"/>
-      <c r="V18" s="380" t="n"/>
+      <c r="S18" s="563" t="n"/>
+      <c r="T18" s="563" t="n"/>
+      <c r="U18" s="563" t="n"/>
+      <c r="V18" s="563" t="n"/>
       <c r="W18" s="502" t="n"/>
-      <c r="X18" s="380" t="n"/>
-      <c r="Y18" s="380" t="n"/>
-      <c r="Z18" s="380" t="n"/>
+      <c r="X18" s="563" t="n"/>
+      <c r="Y18" s="563" t="n"/>
+      <c r="Z18" s="563" t="n"/>
       <c r="AA18" s="502" t="n"/>
-      <c r="AB18" s="380" t="n"/>
-      <c r="AC18" s="380" t="n"/>
-      <c r="AD18" s="380" t="n"/>
+      <c r="AB18" s="563" t="n"/>
+      <c r="AC18" s="563" t="n"/>
+      <c r="AD18" s="563" t="n"/>
       <c r="AE18" s="502" t="n"/>
-      <c r="AF18" s="380" t="n"/>
-      <c r="AG18" s="380" t="n"/>
-      <c r="AH18" s="380" t="n"/>
+      <c r="AF18" s="563" t="n"/>
+      <c r="AG18" s="563" t="n"/>
+      <c r="AH18" s="563" t="n"/>
       <c r="AI18" s="502" t="n"/>
-      <c r="AJ18" s="380" t="n"/>
-      <c r="AK18" s="380" t="n"/>
-      <c r="AL18" s="380" t="n"/>
-      <c r="AM18" s="380" t="n"/>
+      <c r="AJ18" s="563" t="n"/>
+      <c r="AK18" s="563" t="n"/>
+      <c r="AL18" s="563" t="n"/>
+      <c r="AM18" s="563" t="n"/>
       <c r="AN18" s="502" t="n"/>
-      <c r="AO18" s="380" t="n"/>
-      <c r="AP18" s="380" t="n"/>
-      <c r="AQ18" s="380" t="n"/>
+      <c r="AO18" s="563" t="n"/>
+      <c r="AP18" s="563" t="n"/>
+      <c r="AQ18" s="563" t="n"/>
       <c r="AR18" s="502" t="n"/>
-      <c r="AS18" s="380" t="n"/>
-      <c r="AT18" s="380" t="n"/>
-      <c r="AU18" s="380" t="n"/>
+      <c r="AS18" s="563" t="n"/>
+      <c r="AT18" s="563" t="n"/>
+      <c r="AU18" s="563" t="n"/>
       <c r="AV18" s="502" t="n"/>
-      <c r="AW18" s="380" t="n"/>
-      <c r="AX18" s="380" t="n"/>
-      <c r="AY18" s="380" t="n"/>
-      <c r="AZ18" s="502" t="n"/>
-      <c r="BA18" s="380" t="n"/>
-      <c r="BB18" s="380" t="n"/>
-      <c r="BC18" s="380" t="n"/>
-      <c r="BD18" s="491" t="n"/>
+      <c r="AW18" s="563" t="n"/>
+      <c r="AX18" s="563" t="n"/>
+      <c r="AY18" s="563" t="n"/>
+      <c r="AZ18" s="571" t="n"/>
+      <c r="BA18" s="563" t="n"/>
+      <c r="BB18" s="563" t="n"/>
+      <c r="BC18" s="563" t="n"/>
+      <c r="BD18" s="565" t="n"/>
     </row>
     <row r="19" ht="20" customHeight="1">
       <c r="A19" s="501" t="n"/>
-      <c r="B19" s="349" t="n"/>
+      <c r="B19" s="408" t="n"/>
       <c r="C19" s="502" t="n"/>
-      <c r="D19" s="380" t="n"/>
-      <c r="E19" s="380" t="n"/>
-      <c r="F19" s="380" t="n"/>
-      <c r="G19" s="380" t="n"/>
+      <c r="D19" s="563" t="n"/>
+      <c r="E19" s="563" t="n"/>
+      <c r="F19" s="563" t="n"/>
+      <c r="G19" s="563" t="n"/>
       <c r="H19" s="502" t="n"/>
-      <c r="I19" s="380" t="n"/>
-      <c r="J19" s="380" t="n"/>
-      <c r="K19" s="380" t="n"/>
-      <c r="L19" s="380" t="n"/>
+      <c r="I19" s="563" t="n"/>
+      <c r="J19" s="563" t="n"/>
+      <c r="K19" s="563" t="n"/>
+      <c r="L19" s="563" t="n"/>
       <c r="M19" s="502" t="n"/>
-      <c r="N19" s="380" t="n"/>
-      <c r="O19" s="380" t="n"/>
-      <c r="P19" s="380" t="n"/>
-      <c r="Q19" s="380" t="n"/>
+      <c r="N19" s="563" t="n"/>
+      <c r="O19" s="563" t="n"/>
+      <c r="P19" s="563" t="n"/>
+      <c r="Q19" s="563" t="n"/>
       <c r="R19" s="502" t="n"/>
-      <c r="S19" s="380" t="n"/>
-      <c r="T19" s="380" t="n"/>
-      <c r="U19" s="380" t="n"/>
-      <c r="V19" s="380" t="n"/>
+      <c r="S19" s="563" t="n"/>
+      <c r="T19" s="563" t="n"/>
+      <c r="U19" s="563" t="n"/>
+      <c r="V19" s="563" t="n"/>
       <c r="W19" s="502" t="n"/>
-      <c r="X19" s="380" t="n"/>
-      <c r="Y19" s="380" t="n"/>
-      <c r="Z19" s="380" t="n"/>
+      <c r="X19" s="563" t="n"/>
+      <c r="Y19" s="563" t="n"/>
+      <c r="Z19" s="563" t="n"/>
       <c r="AA19" s="502" t="n"/>
-      <c r="AB19" s="380" t="n"/>
-      <c r="AC19" s="380" t="n"/>
-      <c r="AD19" s="380" t="n"/>
+      <c r="AB19" s="563" t="n"/>
+      <c r="AC19" s="563" t="n"/>
+      <c r="AD19" s="563" t="n"/>
       <c r="AE19" s="502" t="n"/>
-      <c r="AF19" s="380" t="n"/>
-      <c r="AG19" s="380" t="n"/>
-      <c r="AH19" s="380" t="n"/>
+      <c r="AF19" s="563" t="n"/>
+      <c r="AG19" s="563" t="n"/>
+      <c r="AH19" s="563" t="n"/>
       <c r="AI19" s="502" t="n"/>
-      <c r="AJ19" s="380" t="n"/>
-      <c r="AK19" s="380" t="n"/>
-      <c r="AL19" s="380" t="n"/>
-      <c r="AM19" s="380" t="n"/>
+      <c r="AJ19" s="563" t="n"/>
+      <c r="AK19" s="563" t="n"/>
+      <c r="AL19" s="563" t="n"/>
+      <c r="AM19" s="563" t="n"/>
       <c r="AN19" s="502" t="n"/>
-      <c r="AO19" s="380" t="n"/>
-      <c r="AP19" s="380" t="n"/>
-      <c r="AQ19" s="380" t="n"/>
+      <c r="AO19" s="563" t="n"/>
+      <c r="AP19" s="563" t="n"/>
+      <c r="AQ19" s="563" t="n"/>
       <c r="AR19" s="502" t="n"/>
-      <c r="AS19" s="380" t="n"/>
-      <c r="AT19" s="380" t="n"/>
-      <c r="AU19" s="380" t="n"/>
+      <c r="AS19" s="563" t="n"/>
+      <c r="AT19" s="563" t="n"/>
+      <c r="AU19" s="563" t="n"/>
       <c r="AV19" s="502" t="n"/>
-      <c r="AW19" s="380" t="n"/>
-      <c r="AX19" s="380" t="n"/>
-      <c r="AY19" s="380" t="n"/>
-      <c r="AZ19" s="502" t="n"/>
-      <c r="BA19" s="380" t="n"/>
-      <c r="BB19" s="380" t="n"/>
-      <c r="BC19" s="380" t="n"/>
-      <c r="BD19" s="491" t="n"/>
+      <c r="AW19" s="563" t="n"/>
+      <c r="AX19" s="563" t="n"/>
+      <c r="AY19" s="563" t="n"/>
+      <c r="AZ19" s="571" t="n"/>
+      <c r="BA19" s="563" t="n"/>
+      <c r="BB19" s="563" t="n"/>
+      <c r="BC19" s="563" t="n"/>
+      <c r="BD19" s="565" t="n"/>
     </row>
     <row r="20" ht="20" customHeight="1">
       <c r="A20" s="501" t="n"/>
-      <c r="B20" s="349" t="n"/>
+      <c r="B20" s="408" t="n"/>
       <c r="C20" s="502" t="n"/>
-      <c r="D20" s="380" t="n"/>
-      <c r="E20" s="380" t="n"/>
-      <c r="F20" s="380" t="n"/>
-      <c r="G20" s="380" t="n"/>
+      <c r="D20" s="563" t="n"/>
+      <c r="E20" s="563" t="n"/>
+      <c r="F20" s="563" t="n"/>
+      <c r="G20" s="563" t="n"/>
       <c r="H20" s="502" t="n"/>
-      <c r="I20" s="380" t="n"/>
-      <c r="J20" s="380" t="n"/>
-      <c r="K20" s="380" t="n"/>
-      <c r="L20" s="380" t="n"/>
+      <c r="I20" s="563" t="n"/>
+      <c r="J20" s="563" t="n"/>
+      <c r="K20" s="563" t="n"/>
+      <c r="L20" s="563" t="n"/>
       <c r="M20" s="502" t="n"/>
-      <c r="N20" s="380" t="n"/>
-      <c r="O20" s="380" t="n"/>
-      <c r="P20" s="380" t="n"/>
-      <c r="Q20" s="380" t="n"/>
+      <c r="N20" s="563" t="n"/>
+      <c r="O20" s="563" t="n"/>
+      <c r="P20" s="563" t="n"/>
+      <c r="Q20" s="563" t="n"/>
       <c r="R20" s="502" t="n"/>
-      <c r="S20" s="380" t="n"/>
-      <c r="T20" s="380" t="n"/>
-      <c r="U20" s="380" t="n"/>
-      <c r="V20" s="380" t="n"/>
+      <c r="S20" s="563" t="n"/>
+      <c r="T20" s="563" t="n"/>
+      <c r="U20" s="563" t="n"/>
+      <c r="V20" s="563" t="n"/>
       <c r="W20" s="502" t="n"/>
-      <c r="X20" s="380" t="n"/>
-      <c r="Y20" s="380" t="n"/>
-      <c r="Z20" s="380" t="n"/>
+      <c r="X20" s="563" t="n"/>
+      <c r="Y20" s="563" t="n"/>
+      <c r="Z20" s="563" t="n"/>
       <c r="AA20" s="502" t="n"/>
-      <c r="AB20" s="380" t="n"/>
-      <c r="AC20" s="380" t="n"/>
-      <c r="AD20" s="380" t="n"/>
+      <c r="AB20" s="563" t="n"/>
+      <c r="AC20" s="563" t="n"/>
+      <c r="AD20" s="563" t="n"/>
       <c r="AE20" s="502" t="n"/>
-      <c r="AF20" s="380" t="n"/>
-      <c r="AG20" s="380" t="n"/>
-      <c r="AH20" s="380" t="n"/>
+      <c r="AF20" s="563" t="n"/>
+      <c r="AG20" s="563" t="n"/>
+      <c r="AH20" s="563" t="n"/>
       <c r="AI20" s="502" t="n"/>
-      <c r="AJ20" s="380" t="n"/>
-      <c r="AK20" s="380" t="n"/>
-      <c r="AL20" s="380" t="n"/>
-      <c r="AM20" s="380" t="n"/>
+      <c r="AJ20" s="563" t="n"/>
+      <c r="AK20" s="563" t="n"/>
+      <c r="AL20" s="563" t="n"/>
+      <c r="AM20" s="563" t="n"/>
       <c r="AN20" s="502" t="n"/>
-      <c r="AO20" s="380" t="n"/>
-      <c r="AP20" s="380" t="n"/>
-      <c r="AQ20" s="380" t="n"/>
+      <c r="AO20" s="563" t="n"/>
+      <c r="AP20" s="563" t="n"/>
+      <c r="AQ20" s="563" t="n"/>
       <c r="AR20" s="502" t="n"/>
-      <c r="AS20" s="380" t="n"/>
-      <c r="AT20" s="380" t="n"/>
-      <c r="AU20" s="380" t="n"/>
+      <c r="AS20" s="563" t="n"/>
+      <c r="AT20" s="563" t="n"/>
+      <c r="AU20" s="563" t="n"/>
       <c r="AV20" s="502" t="n"/>
-      <c r="AW20" s="380" t="n"/>
-      <c r="AX20" s="380" t="n"/>
-      <c r="AY20" s="380" t="n"/>
-      <c r="AZ20" s="502" t="n"/>
-      <c r="BA20" s="380" t="n"/>
-      <c r="BB20" s="380" t="n"/>
-      <c r="BC20" s="380" t="n"/>
-      <c r="BD20" s="491" t="n"/>
+      <c r="AW20" s="563" t="n"/>
+      <c r="AX20" s="563" t="n"/>
+      <c r="AY20" s="563" t="n"/>
+      <c r="AZ20" s="571" t="n"/>
+      <c r="BA20" s="563" t="n"/>
+      <c r="BB20" s="563" t="n"/>
+      <c r="BC20" s="563" t="n"/>
+      <c r="BD20" s="565" t="n"/>
     </row>
     <row r="21" ht="20" customHeight="1">
       <c r="A21" s="501" t="n"/>
-      <c r="B21" s="349" t="n"/>
+      <c r="B21" s="408" t="n"/>
       <c r="C21" s="502" t="n"/>
-      <c r="D21" s="380" t="n"/>
-      <c r="E21" s="380" t="n"/>
-      <c r="F21" s="380" t="n"/>
-      <c r="G21" s="380" t="n"/>
+      <c r="D21" s="563" t="n"/>
+      <c r="E21" s="563" t="n"/>
+      <c r="F21" s="563" t="n"/>
+      <c r="G21" s="563" t="n"/>
       <c r="H21" s="502" t="n"/>
-      <c r="I21" s="380" t="n"/>
-      <c r="J21" s="380" t="n"/>
-      <c r="K21" s="380" t="n"/>
-      <c r="L21" s="380" t="n"/>
+      <c r="I21" s="563" t="n"/>
+      <c r="J21" s="563" t="n"/>
+      <c r="K21" s="563" t="n"/>
+      <c r="L21" s="563" t="n"/>
       <c r="M21" s="502" t="n"/>
-      <c r="N21" s="380" t="n"/>
-      <c r="O21" s="380" t="n"/>
-      <c r="P21" s="380" t="n"/>
-      <c r="Q21" s="380" t="n"/>
+      <c r="N21" s="563" t="n"/>
+      <c r="O21" s="563" t="n"/>
+      <c r="P21" s="563" t="n"/>
+      <c r="Q21" s="563" t="n"/>
       <c r="R21" s="502" t="n"/>
-      <c r="S21" s="380" t="n"/>
-      <c r="T21" s="380" t="n"/>
-      <c r="U21" s="380" t="n"/>
-      <c r="V21" s="380" t="n"/>
+      <c r="S21" s="563" t="n"/>
+      <c r="T21" s="563" t="n"/>
+      <c r="U21" s="563" t="n"/>
+      <c r="V21" s="563" t="n"/>
       <c r="W21" s="502" t="n"/>
-      <c r="X21" s="380" t="n"/>
-      <c r="Y21" s="380" t="n"/>
-      <c r="Z21" s="380" t="n"/>
+      <c r="X21" s="563" t="n"/>
+      <c r="Y21" s="563" t="n"/>
+      <c r="Z21" s="563" t="n"/>
       <c r="AA21" s="502" t="n"/>
-      <c r="AB21" s="380" t="n"/>
-      <c r="AC21" s="380" t="n"/>
-      <c r="AD21" s="380" t="n"/>
+      <c r="AB21" s="563" t="n"/>
+      <c r="AC21" s="563" t="n"/>
+      <c r="AD21" s="563" t="n"/>
       <c r="AE21" s="502" t="n"/>
-      <c r="AF21" s="380" t="n"/>
-      <c r="AG21" s="380" t="n"/>
-      <c r="AH21" s="380" t="n"/>
+      <c r="AF21" s="563" t="n"/>
+      <c r="AG21" s="563" t="n"/>
+      <c r="AH21" s="563" t="n"/>
       <c r="AI21" s="502" t="n"/>
-      <c r="AJ21" s="380" t="n"/>
-      <c r="AK21" s="380" t="n"/>
-      <c r="AL21" s="380" t="n"/>
-      <c r="AM21" s="380" t="n"/>
+      <c r="AJ21" s="563" t="n"/>
+      <c r="AK21" s="563" t="n"/>
+      <c r="AL21" s="563" t="n"/>
+      <c r="AM21" s="563" t="n"/>
       <c r="AN21" s="502" t="n"/>
-      <c r="AO21" s="380" t="n"/>
-      <c r="AP21" s="380" t="n"/>
-      <c r="AQ21" s="380" t="n"/>
+      <c r="AO21" s="563" t="n"/>
+      <c r="AP21" s="563" t="n"/>
+      <c r="AQ21" s="563" t="n"/>
       <c r="AR21" s="502" t="n"/>
-      <c r="AS21" s="380" t="n"/>
-      <c r="AT21" s="380" t="n"/>
-      <c r="AU21" s="380" t="n"/>
+      <c r="AS21" s="563" t="n"/>
+      <c r="AT21" s="563" t="n"/>
+      <c r="AU21" s="563" t="n"/>
       <c r="AV21" s="502" t="n"/>
-      <c r="AW21" s="380" t="n"/>
-      <c r="AX21" s="380" t="n"/>
-      <c r="AY21" s="380" t="n"/>
-      <c r="AZ21" s="502" t="n"/>
-      <c r="BA21" s="380" t="n"/>
-      <c r="BB21" s="380" t="n"/>
-      <c r="BC21" s="380" t="n"/>
-      <c r="BD21" s="491" t="n"/>
+      <c r="AW21" s="563" t="n"/>
+      <c r="AX21" s="563" t="n"/>
+      <c r="AY21" s="563" t="n"/>
+      <c r="AZ21" s="571" t="n"/>
+      <c r="BA21" s="563" t="n"/>
+      <c r="BB21" s="563" t="n"/>
+      <c r="BC21" s="563" t="n"/>
+      <c r="BD21" s="565" t="n"/>
     </row>
     <row r="22" ht="20" customHeight="1">
       <c r="A22" s="501" t="n"/>
-      <c r="B22" s="349" t="n"/>
+      <c r="B22" s="408" t="n"/>
       <c r="C22" s="502" t="n"/>
-      <c r="D22" s="380" t="n"/>
-      <c r="E22" s="380" t="n"/>
-      <c r="F22" s="380" t="n"/>
-      <c r="G22" s="380" t="n"/>
+      <c r="D22" s="563" t="n"/>
+      <c r="E22" s="563" t="n"/>
+      <c r="F22" s="563" t="n"/>
+      <c r="G22" s="563" t="n"/>
       <c r="H22" s="502" t="n"/>
-      <c r="I22" s="380" t="n"/>
-      <c r="J22" s="380" t="n"/>
-      <c r="K22" s="380" t="n"/>
-      <c r="L22" s="380" t="n"/>
+      <c r="I22" s="563" t="n"/>
+      <c r="J22" s="563" t="n"/>
+      <c r="K22" s="563" t="n"/>
+      <c r="L22" s="563" t="n"/>
       <c r="M22" s="502" t="n"/>
-      <c r="N22" s="380" t="n"/>
-      <c r="O22" s="380" t="n"/>
-      <c r="P22" s="380" t="n"/>
-      <c r="Q22" s="380" t="n"/>
+      <c r="N22" s="563" t="n"/>
+      <c r="O22" s="563" t="n"/>
+      <c r="P22" s="563" t="n"/>
+      <c r="Q22" s="563" t="n"/>
       <c r="R22" s="502" t="n"/>
-      <c r="S22" s="380" t="n"/>
-      <c r="T22" s="380" t="n"/>
-      <c r="U22" s="380" t="n"/>
-      <c r="V22" s="380" t="n"/>
+      <c r="S22" s="563" t="n"/>
+      <c r="T22" s="563" t="n"/>
+      <c r="U22" s="563" t="n"/>
+      <c r="V22" s="563" t="n"/>
       <c r="W22" s="502" t="n"/>
-      <c r="X22" s="380" t="n"/>
-      <c r="Y22" s="380" t="n"/>
-      <c r="Z22" s="380" t="n"/>
+      <c r="X22" s="563" t="n"/>
+      <c r="Y22" s="563" t="n"/>
+      <c r="Z22" s="563" t="n"/>
       <c r="AA22" s="502" t="n"/>
-      <c r="AB22" s="380" t="n"/>
-      <c r="AC22" s="380" t="n"/>
-      <c r="AD22" s="380" t="n"/>
+      <c r="AB22" s="563" t="n"/>
+      <c r="AC22" s="563" t="n"/>
+      <c r="AD22" s="563" t="n"/>
       <c r="AE22" s="502" t="n"/>
-      <c r="AF22" s="380" t="n"/>
-      <c r="AG22" s="380" t="n"/>
-      <c r="AH22" s="380" t="n"/>
+      <c r="AF22" s="563" t="n"/>
+      <c r="AG22" s="563" t="n"/>
+      <c r="AH22" s="563" t="n"/>
       <c r="AI22" s="502" t="n"/>
-      <c r="AJ22" s="380" t="n"/>
-      <c r="AK22" s="380" t="n"/>
-      <c r="AL22" s="380" t="n"/>
-      <c r="AM22" s="380" t="n"/>
+      <c r="AJ22" s="563" t="n"/>
+      <c r="AK22" s="563" t="n"/>
+      <c r="AL22" s="563" t="n"/>
+      <c r="AM22" s="563" t="n"/>
       <c r="AN22" s="502" t="n"/>
-      <c r="AO22" s="380" t="n"/>
-      <c r="AP22" s="380" t="n"/>
-      <c r="AQ22" s="380" t="n"/>
+      <c r="AO22" s="563" t="n"/>
+      <c r="AP22" s="563" t="n"/>
+      <c r="AQ22" s="563" t="n"/>
       <c r="AR22" s="502" t="n"/>
-      <c r="AS22" s="380" t="n"/>
-      <c r="AT22" s="380" t="n"/>
-      <c r="AU22" s="380" t="n"/>
+      <c r="AS22" s="563" t="n"/>
+      <c r="AT22" s="563" t="n"/>
+      <c r="AU22" s="563" t="n"/>
       <c r="AV22" s="502" t="n"/>
-      <c r="AW22" s="380" t="n"/>
-      <c r="AX22" s="380" t="n"/>
-      <c r="AY22" s="380" t="n"/>
-      <c r="AZ22" s="502" t="n"/>
-      <c r="BA22" s="380" t="n"/>
-      <c r="BB22" s="380" t="n"/>
-      <c r="BC22" s="380" t="n"/>
-      <c r="BD22" s="491" t="n"/>
+      <c r="AW22" s="563" t="n"/>
+      <c r="AX22" s="563" t="n"/>
+      <c r="AY22" s="563" t="n"/>
+      <c r="AZ22" s="571" t="n"/>
+      <c r="BA22" s="563" t="n"/>
+      <c r="BB22" s="563" t="n"/>
+      <c r="BC22" s="563" t="n"/>
+      <c r="BD22" s="565" t="n"/>
     </row>
     <row r="23" ht="20" customHeight="1">
       <c r="A23" s="501" t="n"/>
-      <c r="B23" s="349" t="n"/>
+      <c r="B23" s="408" t="n"/>
       <c r="C23" s="502" t="n"/>
-      <c r="D23" s="380" t="n"/>
-      <c r="E23" s="380" t="n"/>
-      <c r="F23" s="380" t="n"/>
-      <c r="G23" s="380" t="n"/>
+      <c r="D23" s="563" t="n"/>
+      <c r="E23" s="563" t="n"/>
+      <c r="F23" s="563" t="n"/>
+      <c r="G23" s="563" t="n"/>
       <c r="H23" s="502" t="n"/>
-      <c r="I23" s="380" t="n"/>
-      <c r="J23" s="380" t="n"/>
-      <c r="K23" s="380" t="n"/>
-      <c r="L23" s="380" t="n"/>
+      <c r="I23" s="563" t="n"/>
+      <c r="J23" s="563" t="n"/>
+      <c r="K23" s="563" t="n"/>
+      <c r="L23" s="563" t="n"/>
       <c r="M23" s="502" t="n"/>
-      <c r="N23" s="380" t="n"/>
-      <c r="O23" s="380" t="n"/>
-      <c r="P23" s="380" t="n"/>
-      <c r="Q23" s="380" t="n"/>
+      <c r="N23" s="563" t="n"/>
+      <c r="O23" s="563" t="n"/>
+      <c r="P23" s="563" t="n"/>
+      <c r="Q23" s="563" t="n"/>
       <c r="R23" s="502" t="n"/>
-      <c r="S23" s="380" t="n"/>
-      <c r="T23" s="380" t="n"/>
-      <c r="U23" s="380" t="n"/>
-      <c r="V23" s="380" t="n"/>
+      <c r="S23" s="563" t="n"/>
+      <c r="T23" s="563" t="n"/>
+      <c r="U23" s="563" t="n"/>
+      <c r="V23" s="563" t="n"/>
       <c r="W23" s="502" t="n"/>
-      <c r="X23" s="380" t="n"/>
-      <c r="Y23" s="380" t="n"/>
-      <c r="Z23" s="380" t="n"/>
+      <c r="X23" s="563" t="n"/>
+      <c r="Y23" s="563" t="n"/>
+      <c r="Z23" s="563" t="n"/>
       <c r="AA23" s="502" t="n"/>
-      <c r="AB23" s="380" t="n"/>
-      <c r="AC23" s="380" t="n"/>
-      <c r="AD23" s="380" t="n"/>
+      <c r="AB23" s="563" t="n"/>
+      <c r="AC23" s="563" t="n"/>
+      <c r="AD23" s="563" t="n"/>
       <c r="AE23" s="502" t="n"/>
-      <c r="AF23" s="380" t="n"/>
-      <c r="AG23" s="380" t="n"/>
-      <c r="AH23" s="380" t="n"/>
+      <c r="AF23" s="563" t="n"/>
+      <c r="AG23" s="563" t="n"/>
+      <c r="AH23" s="563" t="n"/>
       <c r="AI23" s="502" t="n"/>
-      <c r="AJ23" s="380" t="n"/>
-      <c r="AK23" s="380" t="n"/>
-      <c r="AL23" s="380" t="n"/>
-      <c r="AM23" s="380" t="n"/>
+      <c r="AJ23" s="563" t="n"/>
+      <c r="AK23" s="563" t="n"/>
+      <c r="AL23" s="563" t="n"/>
+      <c r="AM23" s="563" t="n"/>
       <c r="AN23" s="502" t="n"/>
-      <c r="AO23" s="380" t="n"/>
-      <c r="AP23" s="380" t="n"/>
-      <c r="AQ23" s="380" t="n"/>
+      <c r="AO23" s="563" t="n"/>
+      <c r="AP23" s="563" t="n"/>
+      <c r="AQ23" s="563" t="n"/>
       <c r="AR23" s="502" t="n"/>
-      <c r="AS23" s="380" t="n"/>
-      <c r="AT23" s="380" t="n"/>
-      <c r="AU23" s="380" t="n"/>
+      <c r="AS23" s="563" t="n"/>
+      <c r="AT23" s="563" t="n"/>
+      <c r="AU23" s="563" t="n"/>
       <c r="AV23" s="502" t="n"/>
-      <c r="AW23" s="380" t="n"/>
-      <c r="AX23" s="380" t="n"/>
-      <c r="AY23" s="380" t="n"/>
-      <c r="AZ23" s="502" t="n"/>
-      <c r="BA23" s="380" t="n"/>
-      <c r="BB23" s="380" t="n"/>
-      <c r="BC23" s="380" t="n"/>
-      <c r="BD23" s="491" t="n"/>
+      <c r="AW23" s="563" t="n"/>
+      <c r="AX23" s="563" t="n"/>
+      <c r="AY23" s="563" t="n"/>
+      <c r="AZ23" s="571" t="n"/>
+      <c r="BA23" s="563" t="n"/>
+      <c r="BB23" s="563" t="n"/>
+      <c r="BC23" s="563" t="n"/>
+      <c r="BD23" s="565" t="n"/>
     </row>
     <row r="24" ht="20" customHeight="1">
       <c r="A24" s="501" t="n"/>
-      <c r="B24" s="349" t="n"/>
+      <c r="B24" s="408" t="n"/>
       <c r="C24" s="502" t="n"/>
-      <c r="D24" s="380" t="n"/>
-      <c r="E24" s="380" t="n"/>
-      <c r="F24" s="380" t="n"/>
-      <c r="G24" s="380" t="n"/>
+      <c r="D24" s="563" t="n"/>
+      <c r="E24" s="563" t="n"/>
+      <c r="F24" s="563" t="n"/>
+      <c r="G24" s="563" t="n"/>
       <c r="H24" s="502" t="n"/>
-      <c r="I24" s="380" t="n"/>
-      <c r="J24" s="380" t="n"/>
-      <c r="K24" s="380" t="n"/>
-      <c r="L24" s="380" t="n"/>
+      <c r="I24" s="563" t="n"/>
+      <c r="J24" s="563" t="n"/>
+      <c r="K24" s="563" t="n"/>
+      <c r="L24" s="563" t="n"/>
       <c r="M24" s="502" t="n"/>
-      <c r="N24" s="380" t="n"/>
-      <c r="O24" s="380" t="n"/>
-      <c r="P24" s="380" t="n"/>
-      <c r="Q24" s="380" t="n"/>
+      <c r="N24" s="563" t="n"/>
+      <c r="O24" s="563" t="n"/>
+      <c r="P24" s="563" t="n"/>
+      <c r="Q24" s="563" t="n"/>
       <c r="R24" s="502" t="n"/>
-      <c r="S24" s="380" t="n"/>
-      <c r="T24" s="380" t="n"/>
-      <c r="U24" s="380" t="n"/>
-      <c r="V24" s="380" t="n"/>
+      <c r="S24" s="563" t="n"/>
+      <c r="T24" s="563" t="n"/>
+      <c r="U24" s="563" t="n"/>
+      <c r="V24" s="563" t="n"/>
       <c r="W24" s="502" t="n"/>
-      <c r="X24" s="380" t="n"/>
-      <c r="Y24" s="380" t="n"/>
-      <c r="Z24" s="380" t="n"/>
+      <c r="X24" s="563" t="n"/>
+      <c r="Y24" s="563" t="n"/>
+      <c r="Z24" s="563" t="n"/>
       <c r="AA24" s="502" t="n"/>
-      <c r="AB24" s="380" t="n"/>
-      <c r="AC24" s="380" t="n"/>
-      <c r="AD24" s="380" t="n"/>
+      <c r="AB24" s="563" t="n"/>
+      <c r="AC24" s="563" t="n"/>
+      <c r="AD24" s="563" t="n"/>
       <c r="AE24" s="502" t="n"/>
-      <c r="AF24" s="380" t="n"/>
-      <c r="AG24" s="380" t="n"/>
-      <c r="AH24" s="380" t="n"/>
+      <c r="AF24" s="563" t="n"/>
+      <c r="AG24" s="563" t="n"/>
+      <c r="AH24" s="563" t="n"/>
       <c r="AI24" s="502" t="n"/>
-      <c r="AJ24" s="380" t="n"/>
-      <c r="AK24" s="380" t="n"/>
-      <c r="AL24" s="380" t="n"/>
-      <c r="AM24" s="380" t="n"/>
+      <c r="AJ24" s="563" t="n"/>
+      <c r="AK24" s="563" t="n"/>
+      <c r="AL24" s="563" t="n"/>
+      <c r="AM24" s="563" t="n"/>
       <c r="AN24" s="502" t="n"/>
-      <c r="AO24" s="380" t="n"/>
-      <c r="AP24" s="380" t="n"/>
-      <c r="AQ24" s="380" t="n"/>
+      <c r="AO24" s="563" t="n"/>
+      <c r="AP24" s="563" t="n"/>
+      <c r="AQ24" s="563" t="n"/>
       <c r="AR24" s="502" t="n"/>
-      <c r="AS24" s="380" t="n"/>
-      <c r="AT24" s="380" t="n"/>
-      <c r="AU24" s="380" t="n"/>
+      <c r="AS24" s="563" t="n"/>
+      <c r="AT24" s="563" t="n"/>
+      <c r="AU24" s="563" t="n"/>
       <c r="AV24" s="502" t="n"/>
-      <c r="AW24" s="380" t="n"/>
-      <c r="AX24" s="380" t="n"/>
-      <c r="AY24" s="380" t="n"/>
-      <c r="AZ24" s="502" t="n"/>
-      <c r="BA24" s="380" t="n"/>
-      <c r="BB24" s="380" t="n"/>
-      <c r="BC24" s="380" t="n"/>
-      <c r="BD24" s="491" t="n"/>
+      <c r="AW24" s="563" t="n"/>
+      <c r="AX24" s="563" t="n"/>
+      <c r="AY24" s="563" t="n"/>
+      <c r="AZ24" s="571" t="n"/>
+      <c r="BA24" s="563" t="n"/>
+      <c r="BB24" s="563" t="n"/>
+      <c r="BC24" s="563" t="n"/>
+      <c r="BD24" s="565" t="n"/>
     </row>
     <row r="25" ht="20" customHeight="1">
       <c r="A25" s="501" t="n"/>
-      <c r="B25" s="349" t="n"/>
+      <c r="B25" s="408" t="n"/>
       <c r="C25" s="502" t="n"/>
-      <c r="D25" s="380" t="n"/>
-      <c r="E25" s="380" t="n"/>
-      <c r="F25" s="380" t="n"/>
-      <c r="G25" s="380" t="n"/>
+      <c r="D25" s="563" t="n"/>
+      <c r="E25" s="563" t="n"/>
+      <c r="F25" s="563" t="n"/>
+      <c r="G25" s="563" t="n"/>
       <c r="H25" s="502" t="n"/>
-      <c r="I25" s="380" t="n"/>
-      <c r="J25" s="380" t="n"/>
-      <c r="K25" s="380" t="n"/>
-      <c r="L25" s="380" t="n"/>
+      <c r="I25" s="563" t="n"/>
+      <c r="J25" s="563" t="n"/>
+      <c r="K25" s="563" t="n"/>
+      <c r="L25" s="563" t="n"/>
       <c r="M25" s="502" t="n"/>
-      <c r="N25" s="380" t="n"/>
-      <c r="O25" s="380" t="n"/>
-      <c r="P25" s="380" t="n"/>
-      <c r="Q25" s="380" t="n"/>
+      <c r="N25" s="563" t="n"/>
+      <c r="O25" s="563" t="n"/>
+      <c r="P25" s="563" t="n"/>
+      <c r="Q25" s="563" t="n"/>
       <c r="R25" s="502" t="n"/>
-      <c r="S25" s="380" t="n"/>
-      <c r="T25" s="380" t="n"/>
-      <c r="U25" s="380" t="n"/>
-      <c r="V25" s="380" t="n"/>
+      <c r="S25" s="563" t="n"/>
+      <c r="T25" s="563" t="n"/>
+      <c r="U25" s="563" t="n"/>
+      <c r="V25" s="563" t="n"/>
       <c r="W25" s="502" t="n"/>
-      <c r="X25" s="380" t="n"/>
-      <c r="Y25" s="380" t="n"/>
-      <c r="Z25" s="380" t="n"/>
+      <c r="X25" s="563" t="n"/>
+      <c r="Y25" s="563" t="n"/>
+      <c r="Z25" s="563" t="n"/>
       <c r="AA25" s="502" t="n"/>
-      <c r="AB25" s="380" t="n"/>
-      <c r="AC25" s="380" t="n"/>
-      <c r="AD25" s="380" t="n"/>
+      <c r="AB25" s="563" t="n"/>
+      <c r="AC25" s="563" t="n"/>
+      <c r="AD25" s="563" t="n"/>
       <c r="AE25" s="502" t="n"/>
-      <c r="AF25" s="380" t="n"/>
-      <c r="AG25" s="380" t="n"/>
-      <c r="AH25" s="380" t="n"/>
+      <c r="AF25" s="563" t="n"/>
+      <c r="AG25" s="563" t="n"/>
+      <c r="AH25" s="563" t="n"/>
       <c r="AI25" s="502" t="n"/>
-      <c r="AJ25" s="380" t="n"/>
-      <c r="AK25" s="380" t="n"/>
-      <c r="AL25" s="380" t="n"/>
-      <c r="AM25" s="380" t="n"/>
+      <c r="AJ25" s="563" t="n"/>
+      <c r="AK25" s="563" t="n"/>
+      <c r="AL25" s="563" t="n"/>
+      <c r="AM25" s="563" t="n"/>
       <c r="AN25" s="502" t="n"/>
-      <c r="AO25" s="380" t="n"/>
-      <c r="AP25" s="380" t="n"/>
-      <c r="AQ25" s="380" t="n"/>
+      <c r="AO25" s="563" t="n"/>
+      <c r="AP25" s="563" t="n"/>
+      <c r="AQ25" s="563" t="n"/>
       <c r="AR25" s="502" t="n"/>
-      <c r="AS25" s="380" t="n"/>
-      <c r="AT25" s="380" t="n"/>
-      <c r="AU25" s="380" t="n"/>
+      <c r="AS25" s="563" t="n"/>
+      <c r="AT25" s="563" t="n"/>
+      <c r="AU25" s="563" t="n"/>
       <c r="AV25" s="502" t="n"/>
-      <c r="AW25" s="380" t="n"/>
-      <c r="AX25" s="380" t="n"/>
-      <c r="AY25" s="380" t="n"/>
-      <c r="AZ25" s="502" t="n"/>
-      <c r="BA25" s="380" t="n"/>
-      <c r="BB25" s="380" t="n"/>
-      <c r="BC25" s="380" t="n"/>
-      <c r="BD25" s="491" t="n"/>
+      <c r="AW25" s="563" t="n"/>
+      <c r="AX25" s="563" t="n"/>
+      <c r="AY25" s="563" t="n"/>
+      <c r="AZ25" s="571" t="n"/>
+      <c r="BA25" s="563" t="n"/>
+      <c r="BB25" s="563" t="n"/>
+      <c r="BC25" s="563" t="n"/>
+      <c r="BD25" s="565" t="n"/>
     </row>
     <row r="26" ht="20" customHeight="1">
       <c r="A26" s="503" t="n"/>
-      <c r="B26" s="493" t="n"/>
+      <c r="B26" s="554" t="n"/>
       <c r="C26" s="504" t="n"/>
-      <c r="D26" s="495" t="n"/>
-      <c r="E26" s="495" t="n"/>
-      <c r="F26" s="495" t="n"/>
-      <c r="G26" s="495" t="n"/>
+      <c r="D26" s="566" t="n"/>
+      <c r="E26" s="566" t="n"/>
+      <c r="F26" s="566" t="n"/>
+      <c r="G26" s="566" t="n"/>
       <c r="H26" s="504" t="n"/>
-      <c r="I26" s="495" t="n"/>
-      <c r="J26" s="495" t="n"/>
-      <c r="K26" s="495" t="n"/>
-      <c r="L26" s="495" t="n"/>
+      <c r="I26" s="566" t="n"/>
+      <c r="J26" s="566" t="n"/>
+      <c r="K26" s="566" t="n"/>
+      <c r="L26" s="566" t="n"/>
       <c r="M26" s="504" t="n"/>
-      <c r="N26" s="495" t="n"/>
-      <c r="O26" s="495" t="n"/>
-      <c r="P26" s="495" t="n"/>
-      <c r="Q26" s="495" t="n"/>
+      <c r="N26" s="566" t="n"/>
+      <c r="O26" s="566" t="n"/>
+      <c r="P26" s="566" t="n"/>
+      <c r="Q26" s="566" t="n"/>
       <c r="R26" s="504" t="n"/>
-      <c r="S26" s="495" t="n"/>
-      <c r="T26" s="495" t="n"/>
-      <c r="U26" s="495" t="n"/>
-      <c r="V26" s="495" t="n"/>
+      <c r="S26" s="566" t="n"/>
+      <c r="T26" s="566" t="n"/>
+      <c r="U26" s="566" t="n"/>
+      <c r="V26" s="566" t="n"/>
       <c r="W26" s="504" t="n"/>
-      <c r="X26" s="495" t="n"/>
-      <c r="Y26" s="495" t="n"/>
-      <c r="Z26" s="495" t="n"/>
+      <c r="X26" s="566" t="n"/>
+      <c r="Y26" s="566" t="n"/>
+      <c r="Z26" s="566" t="n"/>
       <c r="AA26" s="504" t="n"/>
-      <c r="AB26" s="495" t="n"/>
-      <c r="AC26" s="495" t="n"/>
-      <c r="AD26" s="495" t="n"/>
+      <c r="AB26" s="566" t="n"/>
+      <c r="AC26" s="566" t="n"/>
+      <c r="AD26" s="566" t="n"/>
       <c r="AE26" s="504" t="n"/>
-      <c r="AF26" s="495" t="n"/>
-      <c r="AG26" s="495" t="n"/>
-      <c r="AH26" s="495" t="n"/>
+      <c r="AF26" s="566" t="n"/>
+      <c r="AG26" s="566" t="n"/>
+      <c r="AH26" s="566" t="n"/>
       <c r="AI26" s="504" t="n"/>
-      <c r="AJ26" s="495" t="n"/>
-      <c r="AK26" s="495" t="n"/>
-      <c r="AL26" s="495" t="n"/>
-      <c r="AM26" s="495" t="n"/>
+      <c r="AJ26" s="566" t="n"/>
+      <c r="AK26" s="566" t="n"/>
+      <c r="AL26" s="566" t="n"/>
+      <c r="AM26" s="566" t="n"/>
       <c r="AN26" s="504" t="n"/>
-      <c r="AO26" s="495" t="n"/>
-      <c r="AP26" s="495" t="n"/>
-      <c r="AQ26" s="495" t="n"/>
+      <c r="AO26" s="566" t="n"/>
+      <c r="AP26" s="566" t="n"/>
+      <c r="AQ26" s="566" t="n"/>
       <c r="AR26" s="504" t="n"/>
-      <c r="AS26" s="495" t="n"/>
-      <c r="AT26" s="495" t="n"/>
-      <c r="AU26" s="495" t="n"/>
+      <c r="AS26" s="566" t="n"/>
+      <c r="AT26" s="566" t="n"/>
+      <c r="AU26" s="566" t="n"/>
       <c r="AV26" s="504" t="n"/>
-      <c r="AW26" s="495" t="n"/>
-      <c r="AX26" s="495" t="n"/>
-      <c r="AY26" s="495" t="n"/>
-      <c r="AZ26" s="504" t="n"/>
-      <c r="BA26" s="495" t="n"/>
-      <c r="BB26" s="495" t="n"/>
-      <c r="BC26" s="495" t="n"/>
-      <c r="BD26" s="497" t="n"/>
+      <c r="AW26" s="566" t="n"/>
+      <c r="AX26" s="566" t="n"/>
+      <c r="AY26" s="566" t="n"/>
+      <c r="AZ26" s="572" t="n"/>
+      <c r="BA26" s="566" t="n"/>
+      <c r="BB26" s="566" t="n"/>
+      <c r="BC26" s="566" t="n"/>
+      <c r="BD26" s="568" t="n"/>
     </row>
     <row r="27" ht="3" customHeight="1">
       <c r="A27" s="386" t="n"/>
@@ -9723,66 +10053,66 @@
       <c r="BD27" s="354" t="n"/>
     </row>
     <row r="28" ht="18" customHeight="1">
-      <c r="A28" s="472" t="inlineStr">
+      <c r="A28" s="558" t="inlineStr">
         <is>
           <t xml:space="preserve">  3. PERIODIC REVIEW / CLOSEOUT</t>
         </is>
       </c>
-      <c r="B28" s="473" t="n"/>
-      <c r="C28" s="473" t="n"/>
-      <c r="D28" s="473" t="n"/>
-      <c r="E28" s="473" t="n"/>
-      <c r="F28" s="473" t="n"/>
-      <c r="G28" s="473" t="n"/>
-      <c r="H28" s="473" t="n"/>
-      <c r="I28" s="473" t="n"/>
-      <c r="J28" s="473" t="n"/>
-      <c r="K28" s="473" t="n"/>
-      <c r="L28" s="473" t="n"/>
-      <c r="M28" s="473" t="n"/>
-      <c r="N28" s="473" t="n"/>
-      <c r="O28" s="473" t="n"/>
-      <c r="P28" s="473" t="n"/>
-      <c r="Q28" s="473" t="n"/>
-      <c r="R28" s="473" t="n"/>
-      <c r="S28" s="473" t="n"/>
-      <c r="T28" s="473" t="n"/>
-      <c r="U28" s="473" t="n"/>
-      <c r="V28" s="473" t="n"/>
-      <c r="W28" s="473" t="n"/>
-      <c r="X28" s="473" t="n"/>
-      <c r="Y28" s="473" t="n"/>
-      <c r="Z28" s="473" t="n"/>
-      <c r="AA28" s="473" t="n"/>
-      <c r="AB28" s="473" t="n"/>
-      <c r="AC28" s="473" t="n"/>
-      <c r="AD28" s="473" t="n"/>
-      <c r="AE28" s="473" t="n"/>
-      <c r="AF28" s="473" t="n"/>
-      <c r="AG28" s="473" t="n"/>
-      <c r="AH28" s="473" t="n"/>
-      <c r="AI28" s="473" t="n"/>
-      <c r="AJ28" s="473" t="n"/>
-      <c r="AK28" s="473" t="n"/>
-      <c r="AL28" s="473" t="n"/>
-      <c r="AM28" s="473" t="n"/>
-      <c r="AN28" s="473" t="n"/>
-      <c r="AO28" s="473" t="n"/>
-      <c r="AP28" s="473" t="n"/>
-      <c r="AQ28" s="473" t="n"/>
-      <c r="AR28" s="473" t="n"/>
-      <c r="AS28" s="473" t="n"/>
-      <c r="AT28" s="473" t="n"/>
-      <c r="AU28" s="473" t="n"/>
-      <c r="AV28" s="473" t="n"/>
-      <c r="AW28" s="473" t="n"/>
-      <c r="AX28" s="473" t="n"/>
-      <c r="AY28" s="473" t="n"/>
-      <c r="AZ28" s="473" t="n"/>
-      <c r="BA28" s="473" t="n"/>
-      <c r="BB28" s="473" t="n"/>
-      <c r="BC28" s="473" t="n"/>
-      <c r="BD28" s="474" t="n"/>
+      <c r="B28" s="535" t="n"/>
+      <c r="C28" s="535" t="n"/>
+      <c r="D28" s="535" t="n"/>
+      <c r="E28" s="535" t="n"/>
+      <c r="F28" s="535" t="n"/>
+      <c r="G28" s="535" t="n"/>
+      <c r="H28" s="535" t="n"/>
+      <c r="I28" s="535" t="n"/>
+      <c r="J28" s="535" t="n"/>
+      <c r="K28" s="535" t="n"/>
+      <c r="L28" s="535" t="n"/>
+      <c r="M28" s="535" t="n"/>
+      <c r="N28" s="535" t="n"/>
+      <c r="O28" s="535" t="n"/>
+      <c r="P28" s="535" t="n"/>
+      <c r="Q28" s="535" t="n"/>
+      <c r="R28" s="535" t="n"/>
+      <c r="S28" s="535" t="n"/>
+      <c r="T28" s="535" t="n"/>
+      <c r="U28" s="535" t="n"/>
+      <c r="V28" s="535" t="n"/>
+      <c r="W28" s="535" t="n"/>
+      <c r="X28" s="535" t="n"/>
+      <c r="Y28" s="535" t="n"/>
+      <c r="Z28" s="535" t="n"/>
+      <c r="AA28" s="535" t="n"/>
+      <c r="AB28" s="535" t="n"/>
+      <c r="AC28" s="535" t="n"/>
+      <c r="AD28" s="535" t="n"/>
+      <c r="AE28" s="535" t="n"/>
+      <c r="AF28" s="535" t="n"/>
+      <c r="AG28" s="535" t="n"/>
+      <c r="AH28" s="535" t="n"/>
+      <c r="AI28" s="535" t="n"/>
+      <c r="AJ28" s="535" t="n"/>
+      <c r="AK28" s="535" t="n"/>
+      <c r="AL28" s="535" t="n"/>
+      <c r="AM28" s="535" t="n"/>
+      <c r="AN28" s="535" t="n"/>
+      <c r="AO28" s="535" t="n"/>
+      <c r="AP28" s="535" t="n"/>
+      <c r="AQ28" s="535" t="n"/>
+      <c r="AR28" s="535" t="n"/>
+      <c r="AS28" s="535" t="n"/>
+      <c r="AT28" s="535" t="n"/>
+      <c r="AU28" s="535" t="n"/>
+      <c r="AV28" s="535" t="n"/>
+      <c r="AW28" s="535" t="n"/>
+      <c r="AX28" s="535" t="n"/>
+      <c r="AY28" s="535" t="n"/>
+      <c r="AZ28" s="535" t="n"/>
+      <c r="BA28" s="535" t="n"/>
+      <c r="BB28" s="535" t="n"/>
+      <c r="BC28" s="535" t="n"/>
+      <c r="BD28" s="559" t="n"/>
     </row>
     <row r="29" ht="26" customHeight="1">
       <c r="A29" s="475" t="inlineStr">
@@ -9790,65 +10120,65 @@
           <t>Periodic Review Date</t>
         </is>
       </c>
-      <c r="B29" s="462" t="n"/>
-      <c r="C29" s="462" t="n"/>
-      <c r="D29" s="462" t="n"/>
-      <c r="E29" s="462" t="n"/>
-      <c r="F29" s="462" t="n"/>
-      <c r="G29" s="462" t="n"/>
-      <c r="H29" s="462" t="n"/>
-      <c r="I29" s="462" t="n"/>
-      <c r="J29" s="462" t="n"/>
+      <c r="B29" s="536" t="n"/>
+      <c r="C29" s="536" t="n"/>
+      <c r="D29" s="536" t="n"/>
+      <c r="E29" s="536" t="n"/>
+      <c r="F29" s="536" t="n"/>
+      <c r="G29" s="536" t="n"/>
+      <c r="H29" s="536" t="n"/>
+      <c r="I29" s="536" t="n"/>
+      <c r="J29" s="536" t="n"/>
       <c r="K29" s="487" t="n"/>
-      <c r="L29" s="488" t="n"/>
-      <c r="M29" s="488" t="n"/>
-      <c r="N29" s="488" t="n"/>
-      <c r="O29" s="488" t="n"/>
-      <c r="P29" s="488" t="n"/>
-      <c r="Q29" s="488" t="n"/>
-      <c r="R29" s="488" t="n"/>
-      <c r="S29" s="488" t="n"/>
-      <c r="T29" s="488" t="n"/>
-      <c r="U29" s="488" t="n"/>
-      <c r="V29" s="488" t="n"/>
-      <c r="W29" s="488" t="n"/>
-      <c r="X29" s="488" t="n"/>
-      <c r="Y29" s="488" t="n"/>
-      <c r="Z29" s="488" t="n"/>
-      <c r="AA29" s="488" t="n"/>
-      <c r="AB29" s="488" t="n"/>
+      <c r="L29" s="560" t="n"/>
+      <c r="M29" s="560" t="n"/>
+      <c r="N29" s="560" t="n"/>
+      <c r="O29" s="560" t="n"/>
+      <c r="P29" s="560" t="n"/>
+      <c r="Q29" s="560" t="n"/>
+      <c r="R29" s="560" t="n"/>
+      <c r="S29" s="560" t="n"/>
+      <c r="T29" s="560" t="n"/>
+      <c r="U29" s="560" t="n"/>
+      <c r="V29" s="560" t="n"/>
+      <c r="W29" s="560" t="n"/>
+      <c r="X29" s="560" t="n"/>
+      <c r="Y29" s="560" t="n"/>
+      <c r="Z29" s="560" t="n"/>
+      <c r="AA29" s="560" t="n"/>
+      <c r="AB29" s="560" t="n"/>
       <c r="AC29" s="477" t="inlineStr">
         <is>
           <t>Reviewer</t>
         </is>
       </c>
-      <c r="AD29" s="462" t="n"/>
-      <c r="AE29" s="462" t="n"/>
-      <c r="AF29" s="462" t="n"/>
-      <c r="AG29" s="462" t="n"/>
-      <c r="AH29" s="462" t="n"/>
-      <c r="AI29" s="462" t="n"/>
-      <c r="AJ29" s="462" t="n"/>
-      <c r="AK29" s="462" t="n"/>
-      <c r="AL29" s="462" t="n"/>
-      <c r="AM29" s="487" t="n"/>
-      <c r="AN29" s="488" t="n"/>
-      <c r="AO29" s="488" t="n"/>
-      <c r="AP29" s="488" t="n"/>
-      <c r="AQ29" s="488" t="n"/>
-      <c r="AR29" s="488" t="n"/>
-      <c r="AS29" s="488" t="n"/>
-      <c r="AT29" s="488" t="n"/>
-      <c r="AU29" s="488" t="n"/>
-      <c r="AV29" s="488" t="n"/>
-      <c r="AW29" s="488" t="n"/>
-      <c r="AX29" s="488" t="n"/>
-      <c r="AY29" s="488" t="n"/>
-      <c r="AZ29" s="488" t="n"/>
-      <c r="BA29" s="488" t="n"/>
-      <c r="BB29" s="488" t="n"/>
-      <c r="BC29" s="488" t="n"/>
-      <c r="BD29" s="489" t="n"/>
+      <c r="AD29" s="536" t="n"/>
+      <c r="AE29" s="536" t="n"/>
+      <c r="AF29" s="536" t="n"/>
+      <c r="AG29" s="536" t="n"/>
+      <c r="AH29" s="536" t="n"/>
+      <c r="AI29" s="536" t="n"/>
+      <c r="AJ29" s="536" t="n"/>
+      <c r="AK29" s="536" t="n"/>
+      <c r="AL29" s="536" t="n"/>
+      <c r="AM29" s="561" t="n"/>
+      <c r="AN29" s="560" t="n"/>
+      <c r="AO29" s="560" t="n"/>
+      <c r="AP29" s="560" t="n"/>
+      <c r="AQ29" s="560" t="n"/>
+      <c r="AR29" s="560" t="n"/>
+      <c r="AS29" s="560" t="n"/>
+      <c r="AT29" s="560" t="n"/>
+      <c r="AU29" s="560" t="n"/>
+      <c r="AV29" s="560" t="n"/>
+      <c r="AW29" s="560" t="n"/>
+      <c r="AX29" s="560" t="n"/>
+      <c r="AY29" s="560" t="n"/>
+      <c r="AZ29" s="560" t="n"/>
+      <c r="BA29" s="560" t="n"/>
+      <c r="BB29" s="560" t="n"/>
+      <c r="BC29" s="560" t="n"/>
+      <c r="BD29" s="562" t="n"/>
     </row>
     <row r="30" ht="20" customHeight="1">
       <c r="A30" s="492" t="inlineStr">
@@ -9856,65 +10186,65 @@
           <t>Open / Escalated Exceptions</t>
         </is>
       </c>
-      <c r="B30" s="493" t="n"/>
-      <c r="C30" s="493" t="n"/>
-      <c r="D30" s="493" t="n"/>
-      <c r="E30" s="493" t="n"/>
-      <c r="F30" s="493" t="n"/>
-      <c r="G30" s="493" t="n"/>
-      <c r="H30" s="493" t="n"/>
-      <c r="I30" s="493" t="n"/>
-      <c r="J30" s="493" t="n"/>
+      <c r="B30" s="554" t="n"/>
+      <c r="C30" s="554" t="n"/>
+      <c r="D30" s="554" t="n"/>
+      <c r="E30" s="554" t="n"/>
+      <c r="F30" s="554" t="n"/>
+      <c r="G30" s="554" t="n"/>
+      <c r="H30" s="554" t="n"/>
+      <c r="I30" s="554" t="n"/>
+      <c r="J30" s="554" t="n"/>
       <c r="K30" s="494" t="n"/>
-      <c r="L30" s="495" t="n"/>
-      <c r="M30" s="495" t="n"/>
-      <c r="N30" s="495" t="n"/>
-      <c r="O30" s="495" t="n"/>
-      <c r="P30" s="495" t="n"/>
-      <c r="Q30" s="495" t="n"/>
-      <c r="R30" s="495" t="n"/>
-      <c r="S30" s="495" t="n"/>
-      <c r="T30" s="495" t="n"/>
-      <c r="U30" s="495" t="n"/>
-      <c r="V30" s="495" t="n"/>
-      <c r="W30" s="495" t="n"/>
-      <c r="X30" s="495" t="n"/>
-      <c r="Y30" s="495" t="n"/>
-      <c r="Z30" s="495" t="n"/>
-      <c r="AA30" s="495" t="n"/>
-      <c r="AB30" s="495" t="n"/>
+      <c r="L30" s="566" t="n"/>
+      <c r="M30" s="566" t="n"/>
+      <c r="N30" s="566" t="n"/>
+      <c r="O30" s="566" t="n"/>
+      <c r="P30" s="566" t="n"/>
+      <c r="Q30" s="566" t="n"/>
+      <c r="R30" s="566" t="n"/>
+      <c r="S30" s="566" t="n"/>
+      <c r="T30" s="566" t="n"/>
+      <c r="U30" s="566" t="n"/>
+      <c r="V30" s="566" t="n"/>
+      <c r="W30" s="566" t="n"/>
+      <c r="X30" s="566" t="n"/>
+      <c r="Y30" s="566" t="n"/>
+      <c r="Z30" s="566" t="n"/>
+      <c r="AA30" s="566" t="n"/>
+      <c r="AB30" s="566" t="n"/>
       <c r="AC30" s="496" t="inlineStr">
         <is>
           <t>Final Status</t>
         </is>
       </c>
-      <c r="AD30" s="493" t="n"/>
-      <c r="AE30" s="493" t="n"/>
-      <c r="AF30" s="493" t="n"/>
-      <c r="AG30" s="493" t="n"/>
-      <c r="AH30" s="493" t="n"/>
-      <c r="AI30" s="493" t="n"/>
-      <c r="AJ30" s="493" t="n"/>
-      <c r="AK30" s="493" t="n"/>
-      <c r="AL30" s="493" t="n"/>
-      <c r="AM30" s="494" t="n"/>
-      <c r="AN30" s="495" t="n"/>
-      <c r="AO30" s="495" t="n"/>
-      <c r="AP30" s="495" t="n"/>
-      <c r="AQ30" s="495" t="n"/>
-      <c r="AR30" s="495" t="n"/>
-      <c r="AS30" s="495" t="n"/>
-      <c r="AT30" s="495" t="n"/>
-      <c r="AU30" s="495" t="n"/>
-      <c r="AV30" s="495" t="n"/>
-      <c r="AW30" s="495" t="n"/>
-      <c r="AX30" s="495" t="n"/>
-      <c r="AY30" s="495" t="n"/>
-      <c r="AZ30" s="495" t="n"/>
-      <c r="BA30" s="495" t="n"/>
-      <c r="BB30" s="495" t="n"/>
-      <c r="BC30" s="495" t="n"/>
-      <c r="BD30" s="497" t="n"/>
+      <c r="AD30" s="554" t="n"/>
+      <c r="AE30" s="554" t="n"/>
+      <c r="AF30" s="554" t="n"/>
+      <c r="AG30" s="554" t="n"/>
+      <c r="AH30" s="554" t="n"/>
+      <c r="AI30" s="554" t="n"/>
+      <c r="AJ30" s="554" t="n"/>
+      <c r="AK30" s="554" t="n"/>
+      <c r="AL30" s="554" t="n"/>
+      <c r="AM30" s="567" t="n"/>
+      <c r="AN30" s="566" t="n"/>
+      <c r="AO30" s="566" t="n"/>
+      <c r="AP30" s="566" t="n"/>
+      <c r="AQ30" s="566" t="n"/>
+      <c r="AR30" s="566" t="n"/>
+      <c r="AS30" s="566" t="n"/>
+      <c r="AT30" s="566" t="n"/>
+      <c r="AU30" s="566" t="n"/>
+      <c r="AV30" s="566" t="n"/>
+      <c r="AW30" s="566" t="n"/>
+      <c r="AX30" s="566" t="n"/>
+      <c r="AY30" s="566" t="n"/>
+      <c r="AZ30" s="566" t="n"/>
+      <c r="BA30" s="566" t="n"/>
+      <c r="BB30" s="566" t="n"/>
+      <c r="BC30" s="566" t="n"/>
+      <c r="BD30" s="568" t="n"/>
     </row>
     <row r="31" ht="3" customHeight="1">
       <c r="A31" s="386" t="n"/>
@@ -9975,66 +10305,66 @@
       <c r="BD31" s="354" t="n"/>
     </row>
     <row r="32" ht="20" customHeight="1">
-      <c r="A32" s="505" t="inlineStr">
+      <c r="A32" s="573" t="inlineStr">
         <is>
           <t>NOTICE: Review face only. Complete row-level entry, filters and frozen-header operations on sheet PO_DATA_LOG. Keep English only, preserve history, record owner and evidence reference, and follow controlled dropdowns / gate rules.</t>
         </is>
       </c>
-      <c r="B32" s="506" t="n"/>
-      <c r="C32" s="506" t="n"/>
-      <c r="D32" s="506" t="n"/>
-      <c r="E32" s="506" t="n"/>
-      <c r="F32" s="506" t="n"/>
-      <c r="G32" s="506" t="n"/>
-      <c r="H32" s="506" t="n"/>
-      <c r="I32" s="506" t="n"/>
-      <c r="J32" s="506" t="n"/>
-      <c r="K32" s="506" t="n"/>
-      <c r="L32" s="506" t="n"/>
-      <c r="M32" s="506" t="n"/>
-      <c r="N32" s="506" t="n"/>
-      <c r="O32" s="506" t="n"/>
-      <c r="P32" s="506" t="n"/>
-      <c r="Q32" s="506" t="n"/>
-      <c r="R32" s="506" t="n"/>
-      <c r="S32" s="506" t="n"/>
-      <c r="T32" s="506" t="n"/>
-      <c r="U32" s="506" t="n"/>
-      <c r="V32" s="506" t="n"/>
-      <c r="W32" s="506" t="n"/>
-      <c r="X32" s="506" t="n"/>
-      <c r="Y32" s="506" t="n"/>
-      <c r="Z32" s="506" t="n"/>
-      <c r="AA32" s="506" t="n"/>
-      <c r="AB32" s="506" t="n"/>
-      <c r="AC32" s="506" t="n"/>
-      <c r="AD32" s="506" t="n"/>
-      <c r="AE32" s="506" t="n"/>
-      <c r="AF32" s="506" t="n"/>
-      <c r="AG32" s="506" t="n"/>
-      <c r="AH32" s="506" t="n"/>
-      <c r="AI32" s="506" t="n"/>
-      <c r="AJ32" s="506" t="n"/>
-      <c r="AK32" s="506" t="n"/>
-      <c r="AL32" s="506" t="n"/>
-      <c r="AM32" s="506" t="n"/>
-      <c r="AN32" s="506" t="n"/>
-      <c r="AO32" s="506" t="n"/>
-      <c r="AP32" s="506" t="n"/>
-      <c r="AQ32" s="506" t="n"/>
-      <c r="AR32" s="506" t="n"/>
-      <c r="AS32" s="506" t="n"/>
-      <c r="AT32" s="506" t="n"/>
-      <c r="AU32" s="506" t="n"/>
-      <c r="AV32" s="506" t="n"/>
-      <c r="AW32" s="506" t="n"/>
-      <c r="AX32" s="506" t="n"/>
-      <c r="AY32" s="506" t="n"/>
-      <c r="AZ32" s="506" t="n"/>
-      <c r="BA32" s="506" t="n"/>
-      <c r="BB32" s="506" t="n"/>
-      <c r="BC32" s="506" t="n"/>
-      <c r="BD32" s="507" t="n"/>
+      <c r="B32" s="535" t="n"/>
+      <c r="C32" s="535" t="n"/>
+      <c r="D32" s="535" t="n"/>
+      <c r="E32" s="535" t="n"/>
+      <c r="F32" s="535" t="n"/>
+      <c r="G32" s="535" t="n"/>
+      <c r="H32" s="535" t="n"/>
+      <c r="I32" s="535" t="n"/>
+      <c r="J32" s="535" t="n"/>
+      <c r="K32" s="535" t="n"/>
+      <c r="L32" s="535" t="n"/>
+      <c r="M32" s="535" t="n"/>
+      <c r="N32" s="535" t="n"/>
+      <c r="O32" s="535" t="n"/>
+      <c r="P32" s="535" t="n"/>
+      <c r="Q32" s="535" t="n"/>
+      <c r="R32" s="535" t="n"/>
+      <c r="S32" s="535" t="n"/>
+      <c r="T32" s="535" t="n"/>
+      <c r="U32" s="535" t="n"/>
+      <c r="V32" s="535" t="n"/>
+      <c r="W32" s="535" t="n"/>
+      <c r="X32" s="535" t="n"/>
+      <c r="Y32" s="535" t="n"/>
+      <c r="Z32" s="535" t="n"/>
+      <c r="AA32" s="535" t="n"/>
+      <c r="AB32" s="535" t="n"/>
+      <c r="AC32" s="535" t="n"/>
+      <c r="AD32" s="535" t="n"/>
+      <c r="AE32" s="535" t="n"/>
+      <c r="AF32" s="535" t="n"/>
+      <c r="AG32" s="535" t="n"/>
+      <c r="AH32" s="535" t="n"/>
+      <c r="AI32" s="535" t="n"/>
+      <c r="AJ32" s="535" t="n"/>
+      <c r="AK32" s="535" t="n"/>
+      <c r="AL32" s="535" t="n"/>
+      <c r="AM32" s="535" t="n"/>
+      <c r="AN32" s="535" t="n"/>
+      <c r="AO32" s="535" t="n"/>
+      <c r="AP32" s="535" t="n"/>
+      <c r="AQ32" s="535" t="n"/>
+      <c r="AR32" s="535" t="n"/>
+      <c r="AS32" s="535" t="n"/>
+      <c r="AT32" s="535" t="n"/>
+      <c r="AU32" s="535" t="n"/>
+      <c r="AV32" s="535" t="n"/>
+      <c r="AW32" s="535" t="n"/>
+      <c r="AX32" s="535" t="n"/>
+      <c r="AY32" s="535" t="n"/>
+      <c r="AZ32" s="535" t="n"/>
+      <c r="BA32" s="535" t="n"/>
+      <c r="BB32" s="535" t="n"/>
+      <c r="BC32" s="535" t="n"/>
+      <c r="BD32" s="559" t="n"/>
     </row>
     <row r="33" ht="17" customHeight="1"/>
     <row r="34" ht="17" customHeight="1"/>
@@ -10286,7 +10616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:CU11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -10512,7 +10842,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AN9"/>
+  <dimension ref="A1:CU9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.33" customWidth="1" min="1" max="1"/>
@@ -10563,12 +10893,12 @@
           <t>Periodic Review Summary</t>
         </is>
       </c>
-      <c r="B1" s="415" t="n"/>
-      <c r="C1" s="415" t="n"/>
-      <c r="D1" s="415" t="n"/>
-      <c r="E1" s="415" t="n"/>
-      <c r="F1" s="415" t="n"/>
-      <c r="G1" s="415" t="n"/>
+      <c r="B1" s="533" t="n"/>
+      <c r="C1" s="533" t="n"/>
+      <c r="D1" s="533" t="n"/>
+      <c r="E1" s="533" t="n"/>
+      <c r="F1" s="533" t="n"/>
+      <c r="G1" s="533" t="n"/>
       <c r="H1" s="509" t="n"/>
       <c r="I1" s="417" t="n"/>
       <c r="J1" s="418" t="n"/>
@@ -10609,12 +10939,6 @@
           <t>Exception-focused PO risk log. Use for promise, cert, traceability, due-date or delivery abnormalities only.</t>
         </is>
       </c>
-      <c r="B2" s="25" t="n"/>
-      <c r="C2" s="25" t="n"/>
-      <c r="D2" s="25" t="n"/>
-      <c r="E2" s="25" t="n"/>
-      <c r="F2" s="25" t="n"/>
-      <c r="G2" s="25" t="n"/>
       <c r="H2" s="440" t="n"/>
       <c r="I2" s="428" t="n"/>
       <c r="J2" s="429" t="n"/>
@@ -11015,7 +11339,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AN13"/>
+  <dimension ref="A1:CU13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.33" customWidth="1" min="1" max="1"/>
@@ -11066,12 +11390,12 @@
           <t>Upstream References / Import Guidance</t>
         </is>
       </c>
-      <c r="B1" s="415" t="n"/>
-      <c r="C1" s="415" t="n"/>
-      <c r="D1" s="415" t="n"/>
-      <c r="E1" s="415" t="n"/>
-      <c r="F1" s="415" t="n"/>
-      <c r="G1" s="415" t="n"/>
+      <c r="B1" s="533" t="n"/>
+      <c r="C1" s="533" t="n"/>
+      <c r="D1" s="533" t="n"/>
+      <c r="E1" s="533" t="n"/>
+      <c r="F1" s="533" t="n"/>
+      <c r="G1" s="533" t="n"/>
       <c r="H1" s="509" t="n"/>
       <c r="I1" s="417" t="n"/>
       <c r="J1" s="418" t="n"/>
@@ -11112,12 +11436,6 @@
           <t>Exception-focused PO risk log. Use for promise, cert, traceability, due-date or delivery abnormalities only.</t>
         </is>
       </c>
-      <c r="B2" s="25" t="n"/>
-      <c r="C2" s="25" t="n"/>
-      <c r="D2" s="25" t="n"/>
-      <c r="E2" s="25" t="n"/>
-      <c r="F2" s="25" t="n"/>
-      <c r="G2" s="25" t="n"/>
       <c r="H2" s="440" t="n"/>
       <c r="I2" s="428" t="n"/>
       <c r="J2" s="429" t="n"/>
@@ -11774,7 +12092,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AN13"/>
+  <dimension ref="A1:CU13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.33" customWidth="1" min="1" max="1"/>

</xml_diff>